<commit_message>
Collections update and a bunch of new stuff
</commit_message>
<xml_diff>
--- a/display/EcoGainsSim_PlybyPly_v6.xlsx
+++ b/display/EcoGainsSim_PlybyPly_v6.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X312"/>
+  <dimension ref="A1:AD312"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.8" customWidth="1" min="1" max="1"/>
@@ -520,6 +520,12 @@
     <col width="7.6" customWidth="1" min="22" max="22"/>
     <col width="7.6" customWidth="1" min="23" max="23"/>
     <col width="7.6" customWidth="1" min="24" max="24"/>
+    <col width="7.6" customWidth="1" min="25" max="25"/>
+    <col width="7.6" customWidth="1" min="26" max="26"/>
+    <col width="7.6" customWidth="1" min="27" max="27"/>
+    <col width="7.6" customWidth="1" min="28" max="28"/>
+    <col width="7.6" customWidth="1" min="29" max="29"/>
+    <col width="7.6" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -950,7 +956,7 @@
     <row r="50">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>12. SPT / SPTx2 are TRACKED since 2026-07-10 (13-resource universe, D16) as event payouts only; season-pass TIER claims are NOT simulated in the session view (window-sim only). COOP Token / Avatar / star-daily rewards remain outside the resource set.</t>
+          <t>12. SPT / SPTx2 are TRACKED since 2026-07-10 (D16) as event payouts only; season-pass TIER claims are NOT simulated in the session view (window-sim only). COOP Token / Avatar remain outside the resource set.</t>
         </is>
       </c>
     </row>
@@ -983,6 +989,12 @@
       <c r="V51" s="2" t="n"/>
       <c r="W51" s="2" t="n"/>
       <c r="X51" s="2" t="n"/>
+      <c r="Y51" s="2" t="n"/>
+      <c r="Z51" s="2" t="n"/>
+      <c r="AA51" s="2" t="n"/>
+      <c r="AB51" s="2" t="n"/>
+      <c r="AC51" s="2" t="n"/>
+      <c r="AD51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="3">
@@ -1012,6 +1024,12 @@
       <c r="V52" s="3" t="n"/>
       <c r="W52" s="3" t="n"/>
       <c r="X52" s="3" t="n"/>
+      <c r="Y52" s="3" t="n"/>
+      <c r="Z52" s="3" t="n"/>
+      <c r="AA52" s="3" t="n"/>
+      <c r="AB52" s="3" t="n"/>
+      <c r="AC52" s="3" t="n"/>
+      <c r="AD52" s="3" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="10" t="n"/>
@@ -1038,6 +1056,12 @@
       <c r="V53" s="10" t="n"/>
       <c r="W53" s="10" t="n"/>
       <c r="X53" s="10" t="n"/>
+      <c r="Y53" s="10" t="n"/>
+      <c r="Z53" s="10" t="n"/>
+      <c r="AA53" s="10" t="n"/>
+      <c r="AB53" s="10" t="n"/>
+      <c r="AC53" s="10" t="n"/>
+      <c r="AD53" s="10" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="n"/>
@@ -1064,6 +1088,12 @@
       <c r="V54" s="10" t="n"/>
       <c r="W54" s="10" t="n"/>
       <c r="X54" s="10" t="n"/>
+      <c r="Y54" s="10" t="n"/>
+      <c r="Z54" s="10" t="n"/>
+      <c r="AA54" s="10" t="n"/>
+      <c r="AB54" s="10" t="n"/>
+      <c r="AC54" s="10" t="n"/>
+      <c r="AD54" s="10" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="10" t="n"/>
@@ -1090,6 +1120,12 @@
       <c r="V55" s="10" t="n"/>
       <c r="W55" s="10" t="n"/>
       <c r="X55" s="10" t="n"/>
+      <c r="Y55" s="10" t="n"/>
+      <c r="Z55" s="10" t="n"/>
+      <c r="AA55" s="10" t="n"/>
+      <c r="AB55" s="10" t="n"/>
+      <c r="AC55" s="10" t="n"/>
+      <c r="AD55" s="10" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="10" t="n"/>
@@ -1116,6 +1152,12 @@
       <c r="V56" s="10" t="n"/>
       <c r="W56" s="10" t="n"/>
       <c r="X56" s="10" t="n"/>
+      <c r="Y56" s="10" t="n"/>
+      <c r="Z56" s="10" t="n"/>
+      <c r="AA56" s="10" t="n"/>
+      <c r="AB56" s="10" t="n"/>
+      <c r="AC56" s="10" t="n"/>
+      <c r="AD56" s="10" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="10" t="n"/>
@@ -1142,6 +1184,12 @@
       <c r="V57" s="10" t="n"/>
       <c r="W57" s="10" t="n"/>
       <c r="X57" s="10" t="n"/>
+      <c r="Y57" s="10" t="n"/>
+      <c r="Z57" s="10" t="n"/>
+      <c r="AA57" s="10" t="n"/>
+      <c r="AB57" s="10" t="n"/>
+      <c r="AC57" s="10" t="n"/>
+      <c r="AD57" s="10" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="10" t="n"/>
@@ -1168,6 +1216,12 @@
       <c r="V58" s="10" t="n"/>
       <c r="W58" s="10" t="n"/>
       <c r="X58" s="10" t="n"/>
+      <c r="Y58" s="10" t="n"/>
+      <c r="Z58" s="10" t="n"/>
+      <c r="AA58" s="10" t="n"/>
+      <c r="AB58" s="10" t="n"/>
+      <c r="AC58" s="10" t="n"/>
+      <c r="AD58" s="10" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="10" t="n"/>
@@ -1194,6 +1248,12 @@
       <c r="V59" s="10" t="n"/>
       <c r="W59" s="10" t="n"/>
       <c r="X59" s="10" t="n"/>
+      <c r="Y59" s="10" t="n"/>
+      <c r="Z59" s="10" t="n"/>
+      <c r="AA59" s="10" t="n"/>
+      <c r="AB59" s="10" t="n"/>
+      <c r="AC59" s="10" t="n"/>
+      <c r="AD59" s="10" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="10" t="n"/>
@@ -1220,6 +1280,12 @@
       <c r="V60" s="10" t="n"/>
       <c r="W60" s="10" t="n"/>
       <c r="X60" s="10" t="n"/>
+      <c r="Y60" s="10" t="n"/>
+      <c r="Z60" s="10" t="n"/>
+      <c r="AA60" s="10" t="n"/>
+      <c r="AB60" s="10" t="n"/>
+      <c r="AC60" s="10" t="n"/>
+      <c r="AD60" s="10" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="10" t="n"/>
@@ -1246,6 +1312,12 @@
       <c r="V61" s="10" t="n"/>
       <c r="W61" s="10" t="n"/>
       <c r="X61" s="10" t="n"/>
+      <c r="Y61" s="10" t="n"/>
+      <c r="Z61" s="10" t="n"/>
+      <c r="AA61" s="10" t="n"/>
+      <c r="AB61" s="10" t="n"/>
+      <c r="AC61" s="10" t="n"/>
+      <c r="AD61" s="10" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="10" t="n"/>
@@ -1272,6 +1344,12 @@
       <c r="V62" s="10" t="n"/>
       <c r="W62" s="10" t="n"/>
       <c r="X62" s="10" t="n"/>
+      <c r="Y62" s="10" t="n"/>
+      <c r="Z62" s="10" t="n"/>
+      <c r="AA62" s="10" t="n"/>
+      <c r="AB62" s="10" t="n"/>
+      <c r="AC62" s="10" t="n"/>
+      <c r="AD62" s="10" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="10" t="n"/>
@@ -1298,6 +1376,12 @@
       <c r="V63" s="10" t="n"/>
       <c r="W63" s="10" t="n"/>
       <c r="X63" s="10" t="n"/>
+      <c r="Y63" s="10" t="n"/>
+      <c r="Z63" s="10" t="n"/>
+      <c r="AA63" s="10" t="n"/>
+      <c r="AB63" s="10" t="n"/>
+      <c r="AC63" s="10" t="n"/>
+      <c r="AD63" s="10" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="10" t="n"/>
@@ -1324,6 +1408,12 @@
       <c r="V64" s="10" t="n"/>
       <c r="W64" s="10" t="n"/>
       <c r="X64" s="10" t="n"/>
+      <c r="Y64" s="10" t="n"/>
+      <c r="Z64" s="10" t="n"/>
+      <c r="AA64" s="10" t="n"/>
+      <c r="AB64" s="10" t="n"/>
+      <c r="AC64" s="10" t="n"/>
+      <c r="AD64" s="10" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="10" t="n"/>
@@ -1350,6 +1440,12 @@
       <c r="V65" s="10" t="n"/>
       <c r="W65" s="10" t="n"/>
       <c r="X65" s="10" t="n"/>
+      <c r="Y65" s="10" t="n"/>
+      <c r="Z65" s="10" t="n"/>
+      <c r="AA65" s="10" t="n"/>
+      <c r="AB65" s="10" t="n"/>
+      <c r="AC65" s="10" t="n"/>
+      <c r="AD65" s="10" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="10" t="n"/>
@@ -1376,6 +1472,12 @@
       <c r="V66" s="10" t="n"/>
       <c r="W66" s="10" t="n"/>
       <c r="X66" s="10" t="n"/>
+      <c r="Y66" s="10" t="n"/>
+      <c r="Z66" s="10" t="n"/>
+      <c r="AA66" s="10" t="n"/>
+      <c r="AB66" s="10" t="n"/>
+      <c r="AC66" s="10" t="n"/>
+      <c r="AD66" s="10" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="10" t="n"/>
@@ -1402,6 +1504,12 @@
       <c r="V67" s="10" t="n"/>
       <c r="W67" s="10" t="n"/>
       <c r="X67" s="10" t="n"/>
+      <c r="Y67" s="10" t="n"/>
+      <c r="Z67" s="10" t="n"/>
+      <c r="AA67" s="10" t="n"/>
+      <c r="AB67" s="10" t="n"/>
+      <c r="AC67" s="10" t="n"/>
+      <c r="AD67" s="10" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="10" t="n"/>
@@ -1428,6 +1536,12 @@
       <c r="V68" s="10" t="n"/>
       <c r="W68" s="10" t="n"/>
       <c r="X68" s="10" t="n"/>
+      <c r="Y68" s="10" t="n"/>
+      <c r="Z68" s="10" t="n"/>
+      <c r="AA68" s="10" t="n"/>
+      <c r="AB68" s="10" t="n"/>
+      <c r="AC68" s="10" t="n"/>
+      <c r="AD68" s="10" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="10" t="n"/>
@@ -1454,6 +1568,12 @@
       <c r="V69" s="10" t="n"/>
       <c r="W69" s="10" t="n"/>
       <c r="X69" s="10" t="n"/>
+      <c r="Y69" s="10" t="n"/>
+      <c r="Z69" s="10" t="n"/>
+      <c r="AA69" s="10" t="n"/>
+      <c r="AB69" s="10" t="n"/>
+      <c r="AC69" s="10" t="n"/>
+      <c r="AD69" s="10" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="10" t="n"/>
@@ -1480,6 +1600,12 @@
       <c r="V70" s="10" t="n"/>
       <c r="W70" s="10" t="n"/>
       <c r="X70" s="10" t="n"/>
+      <c r="Y70" s="10" t="n"/>
+      <c r="Z70" s="10" t="n"/>
+      <c r="AA70" s="10" t="n"/>
+      <c r="AB70" s="10" t="n"/>
+      <c r="AC70" s="10" t="n"/>
+      <c r="AD70" s="10" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="10" t="n"/>
@@ -1506,6 +1632,12 @@
       <c r="V71" s="10" t="n"/>
       <c r="W71" s="10" t="n"/>
       <c r="X71" s="10" t="n"/>
+      <c r="Y71" s="10" t="n"/>
+      <c r="Z71" s="10" t="n"/>
+      <c r="AA71" s="10" t="n"/>
+      <c r="AB71" s="10" t="n"/>
+      <c r="AC71" s="10" t="n"/>
+      <c r="AD71" s="10" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="10" t="n"/>
@@ -1532,6 +1664,12 @@
       <c r="V72" s="10" t="n"/>
       <c r="W72" s="10" t="n"/>
       <c r="X72" s="10" t="n"/>
+      <c r="Y72" s="10" t="n"/>
+      <c r="Z72" s="10" t="n"/>
+      <c r="AA72" s="10" t="n"/>
+      <c r="AB72" s="10" t="n"/>
+      <c r="AC72" s="10" t="n"/>
+      <c r="AD72" s="10" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="10" t="n"/>
@@ -1558,6 +1696,12 @@
       <c r="V73" s="10" t="n"/>
       <c r="W73" s="10" t="n"/>
       <c r="X73" s="10" t="n"/>
+      <c r="Y73" s="10" t="n"/>
+      <c r="Z73" s="10" t="n"/>
+      <c r="AA73" s="10" t="n"/>
+      <c r="AB73" s="10" t="n"/>
+      <c r="AC73" s="10" t="n"/>
+      <c r="AD73" s="10" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="10" t="n"/>
@@ -1584,6 +1728,12 @@
       <c r="V74" s="10" t="n"/>
       <c r="W74" s="10" t="n"/>
       <c r="X74" s="10" t="n"/>
+      <c r="Y74" s="10" t="n"/>
+      <c r="Z74" s="10" t="n"/>
+      <c r="AA74" s="10" t="n"/>
+      <c r="AB74" s="10" t="n"/>
+      <c r="AC74" s="10" t="n"/>
+      <c r="AD74" s="10" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="10" t="n"/>
@@ -1610,6 +1760,12 @@
       <c r="V75" s="10" t="n"/>
       <c r="W75" s="10" t="n"/>
       <c r="X75" s="10" t="n"/>
+      <c r="Y75" s="10" t="n"/>
+      <c r="Z75" s="10" t="n"/>
+      <c r="AA75" s="10" t="n"/>
+      <c r="AB75" s="10" t="n"/>
+      <c r="AC75" s="10" t="n"/>
+      <c r="AD75" s="10" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="10" t="n"/>
@@ -1636,6 +1792,12 @@
       <c r="V76" s="10" t="n"/>
       <c r="W76" s="10" t="n"/>
       <c r="X76" s="10" t="n"/>
+      <c r="Y76" s="10" t="n"/>
+      <c r="Z76" s="10" t="n"/>
+      <c r="AA76" s="10" t="n"/>
+      <c r="AB76" s="10" t="n"/>
+      <c r="AC76" s="10" t="n"/>
+      <c r="AD76" s="10" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="10" t="n"/>
@@ -1662,6 +1824,12 @@
       <c r="V77" s="10" t="n"/>
       <c r="W77" s="10" t="n"/>
       <c r="X77" s="10" t="n"/>
+      <c r="Y77" s="10" t="n"/>
+      <c r="Z77" s="10" t="n"/>
+      <c r="AA77" s="10" t="n"/>
+      <c r="AB77" s="10" t="n"/>
+      <c r="AC77" s="10" t="n"/>
+      <c r="AD77" s="10" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="10" t="n"/>
@@ -1688,6 +1856,12 @@
       <c r="V78" s="10" t="n"/>
       <c r="W78" s="10" t="n"/>
       <c r="X78" s="10" t="n"/>
+      <c r="Y78" s="10" t="n"/>
+      <c r="Z78" s="10" t="n"/>
+      <c r="AA78" s="10" t="n"/>
+      <c r="AB78" s="10" t="n"/>
+      <c r="AC78" s="10" t="n"/>
+      <c r="AD78" s="10" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="10" t="n"/>
@@ -1714,6 +1888,12 @@
       <c r="V79" s="10" t="n"/>
       <c r="W79" s="10" t="n"/>
       <c r="X79" s="10" t="n"/>
+      <c r="Y79" s="10" t="n"/>
+      <c r="Z79" s="10" t="n"/>
+      <c r="AA79" s="10" t="n"/>
+      <c r="AB79" s="10" t="n"/>
+      <c r="AC79" s="10" t="n"/>
+      <c r="AD79" s="10" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="10" t="n"/>
@@ -1740,6 +1920,12 @@
       <c r="V80" s="10" t="n"/>
       <c r="W80" s="10" t="n"/>
       <c r="X80" s="10" t="n"/>
+      <c r="Y80" s="10" t="n"/>
+      <c r="Z80" s="10" t="n"/>
+      <c r="AA80" s="10" t="n"/>
+      <c r="AB80" s="10" t="n"/>
+      <c r="AC80" s="10" t="n"/>
+      <c r="AD80" s="10" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="10" t="n"/>
@@ -1766,6 +1952,12 @@
       <c r="V81" s="10" t="n"/>
       <c r="W81" s="10" t="n"/>
       <c r="X81" s="10" t="n"/>
+      <c r="Y81" s="10" t="n"/>
+      <c r="Z81" s="10" t="n"/>
+      <c r="AA81" s="10" t="n"/>
+      <c r="AB81" s="10" t="n"/>
+      <c r="AC81" s="10" t="n"/>
+      <c r="AD81" s="10" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="10" t="n"/>
@@ -1792,6 +1984,12 @@
       <c r="V82" s="10" t="n"/>
       <c r="W82" s="10" t="n"/>
       <c r="X82" s="10" t="n"/>
+      <c r="Y82" s="10" t="n"/>
+      <c r="Z82" s="10" t="n"/>
+      <c r="AA82" s="10" t="n"/>
+      <c r="AB82" s="10" t="n"/>
+      <c r="AC82" s="10" t="n"/>
+      <c r="AD82" s="10" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="10" t="n"/>
@@ -1818,6 +2016,12 @@
       <c r="V83" s="10" t="n"/>
       <c r="W83" s="10" t="n"/>
       <c r="X83" s="10" t="n"/>
+      <c r="Y83" s="10" t="n"/>
+      <c r="Z83" s="10" t="n"/>
+      <c r="AA83" s="10" t="n"/>
+      <c r="AB83" s="10" t="n"/>
+      <c r="AC83" s="10" t="n"/>
+      <c r="AD83" s="10" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="10" t="n"/>
@@ -1844,6 +2048,12 @@
       <c r="V84" s="10" t="n"/>
       <c r="W84" s="10" t="n"/>
       <c r="X84" s="10" t="n"/>
+      <c r="Y84" s="10" t="n"/>
+      <c r="Z84" s="10" t="n"/>
+      <c r="AA84" s="10" t="n"/>
+      <c r="AB84" s="10" t="n"/>
+      <c r="AC84" s="10" t="n"/>
+      <c r="AD84" s="10" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="10" t="n"/>
@@ -1870,6 +2080,12 @@
       <c r="V85" s="10" t="n"/>
       <c r="W85" s="10" t="n"/>
       <c r="X85" s="10" t="n"/>
+      <c r="Y85" s="10" t="n"/>
+      <c r="Z85" s="10" t="n"/>
+      <c r="AA85" s="10" t="n"/>
+      <c r="AB85" s="10" t="n"/>
+      <c r="AC85" s="10" t="n"/>
+      <c r="AD85" s="10" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="10" t="n"/>
@@ -1896,6 +2112,12 @@
       <c r="V86" s="10" t="n"/>
       <c r="W86" s="10" t="n"/>
       <c r="X86" s="10" t="n"/>
+      <c r="Y86" s="10" t="n"/>
+      <c r="Z86" s="10" t="n"/>
+      <c r="AA86" s="10" t="n"/>
+      <c r="AB86" s="10" t="n"/>
+      <c r="AC86" s="10" t="n"/>
+      <c r="AD86" s="10" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="10" t="n"/>
@@ -1922,6 +2144,12 @@
       <c r="V87" s="10" t="n"/>
       <c r="W87" s="10" t="n"/>
       <c r="X87" s="10" t="n"/>
+      <c r="Y87" s="10" t="n"/>
+      <c r="Z87" s="10" t="n"/>
+      <c r="AA87" s="10" t="n"/>
+      <c r="AB87" s="10" t="n"/>
+      <c r="AC87" s="10" t="n"/>
+      <c r="AD87" s="10" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="10" t="n"/>
@@ -1948,6 +2176,12 @@
       <c r="V88" s="10" t="n"/>
       <c r="W88" s="10" t="n"/>
       <c r="X88" s="10" t="n"/>
+      <c r="Y88" s="10" t="n"/>
+      <c r="Z88" s="10" t="n"/>
+      <c r="AA88" s="10" t="n"/>
+      <c r="AB88" s="10" t="n"/>
+      <c r="AC88" s="10" t="n"/>
+      <c r="AD88" s="10" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="10" t="n"/>
@@ -1974,6 +2208,12 @@
       <c r="V89" s="10" t="n"/>
       <c r="W89" s="10" t="n"/>
       <c r="X89" s="10" t="n"/>
+      <c r="Y89" s="10" t="n"/>
+      <c r="Z89" s="10" t="n"/>
+      <c r="AA89" s="10" t="n"/>
+      <c r="AB89" s="10" t="n"/>
+      <c r="AC89" s="10" t="n"/>
+      <c r="AD89" s="10" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="10" t="n"/>
@@ -2000,6 +2240,12 @@
       <c r="V90" s="10" t="n"/>
       <c r="W90" s="10" t="n"/>
       <c r="X90" s="10" t="n"/>
+      <c r="Y90" s="10" t="n"/>
+      <c r="Z90" s="10" t="n"/>
+      <c r="AA90" s="10" t="n"/>
+      <c r="AB90" s="10" t="n"/>
+      <c r="AC90" s="10" t="n"/>
+      <c r="AD90" s="10" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="10" t="n"/>
@@ -2026,6 +2272,12 @@
       <c r="V91" s="10" t="n"/>
       <c r="W91" s="10" t="n"/>
       <c r="X91" s="10" t="n"/>
+      <c r="Y91" s="10" t="n"/>
+      <c r="Z91" s="10" t="n"/>
+      <c r="AA91" s="10" t="n"/>
+      <c r="AB91" s="10" t="n"/>
+      <c r="AC91" s="10" t="n"/>
+      <c r="AD91" s="10" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="10" t="n"/>
@@ -2052,6 +2304,12 @@
       <c r="V92" s="10" t="n"/>
       <c r="W92" s="10" t="n"/>
       <c r="X92" s="10" t="n"/>
+      <c r="Y92" s="10" t="n"/>
+      <c r="Z92" s="10" t="n"/>
+      <c r="AA92" s="10" t="n"/>
+      <c r="AB92" s="10" t="n"/>
+      <c r="AC92" s="10" t="n"/>
+      <c r="AD92" s="10" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="10" t="n"/>
@@ -2078,6 +2336,12 @@
       <c r="V93" s="10" t="n"/>
       <c r="W93" s="10" t="n"/>
       <c r="X93" s="10" t="n"/>
+      <c r="Y93" s="10" t="n"/>
+      <c r="Z93" s="10" t="n"/>
+      <c r="AA93" s="10" t="n"/>
+      <c r="AB93" s="10" t="n"/>
+      <c r="AC93" s="10" t="n"/>
+      <c r="AD93" s="10" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="10" t="n"/>
@@ -2104,6 +2368,12 @@
       <c r="V94" s="10" t="n"/>
       <c r="W94" s="10" t="n"/>
       <c r="X94" s="10" t="n"/>
+      <c r="Y94" s="10" t="n"/>
+      <c r="Z94" s="10" t="n"/>
+      <c r="AA94" s="10" t="n"/>
+      <c r="AB94" s="10" t="n"/>
+      <c r="AC94" s="10" t="n"/>
+      <c r="AD94" s="10" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="10" t="n"/>
@@ -2130,6 +2400,12 @@
       <c r="V95" s="10" t="n"/>
       <c r="W95" s="10" t="n"/>
       <c r="X95" s="10" t="n"/>
+      <c r="Y95" s="10" t="n"/>
+      <c r="Z95" s="10" t="n"/>
+      <c r="AA95" s="10" t="n"/>
+      <c r="AB95" s="10" t="n"/>
+      <c r="AC95" s="10" t="n"/>
+      <c r="AD95" s="10" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="10" t="n"/>
@@ -2156,6 +2432,12 @@
       <c r="V96" s="10" t="n"/>
       <c r="W96" s="10" t="n"/>
       <c r="X96" s="10" t="n"/>
+      <c r="Y96" s="10" t="n"/>
+      <c r="Z96" s="10" t="n"/>
+      <c r="AA96" s="10" t="n"/>
+      <c r="AB96" s="10" t="n"/>
+      <c r="AC96" s="10" t="n"/>
+      <c r="AD96" s="10" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="10" t="n"/>
@@ -2182,6 +2464,12 @@
       <c r="V97" s="10" t="n"/>
       <c r="W97" s="10" t="n"/>
       <c r="X97" s="10" t="n"/>
+      <c r="Y97" s="10" t="n"/>
+      <c r="Z97" s="10" t="n"/>
+      <c r="AA97" s="10" t="n"/>
+      <c r="AB97" s="10" t="n"/>
+      <c r="AC97" s="10" t="n"/>
+      <c r="AD97" s="10" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="10" t="n"/>
@@ -2208,6 +2496,12 @@
       <c r="V98" s="10" t="n"/>
       <c r="W98" s="10" t="n"/>
       <c r="X98" s="10" t="n"/>
+      <c r="Y98" s="10" t="n"/>
+      <c r="Z98" s="10" t="n"/>
+      <c r="AA98" s="10" t="n"/>
+      <c r="AB98" s="10" t="n"/>
+      <c r="AC98" s="10" t="n"/>
+      <c r="AD98" s="10" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="10" t="n"/>
@@ -2234,6 +2528,12 @@
       <c r="V99" s="10" t="n"/>
       <c r="W99" s="10" t="n"/>
       <c r="X99" s="10" t="n"/>
+      <c r="Y99" s="10" t="n"/>
+      <c r="Z99" s="10" t="n"/>
+      <c r="AA99" s="10" t="n"/>
+      <c r="AB99" s="10" t="n"/>
+      <c r="AC99" s="10" t="n"/>
+      <c r="AD99" s="10" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="10" t="n"/>
@@ -2260,6 +2560,12 @@
       <c r="V100" s="10" t="n"/>
       <c r="W100" s="10" t="n"/>
       <c r="X100" s="10" t="n"/>
+      <c r="Y100" s="10" t="n"/>
+      <c r="Z100" s="10" t="n"/>
+      <c r="AA100" s="10" t="n"/>
+      <c r="AB100" s="10" t="n"/>
+      <c r="AC100" s="10" t="n"/>
+      <c r="AD100" s="10" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="10" t="n"/>
@@ -2286,6 +2592,12 @@
       <c r="V101" s="10" t="n"/>
       <c r="W101" s="10" t="n"/>
       <c r="X101" s="10" t="n"/>
+      <c r="Y101" s="10" t="n"/>
+      <c r="Z101" s="10" t="n"/>
+      <c r="AA101" s="10" t="n"/>
+      <c r="AB101" s="10" t="n"/>
+      <c r="AC101" s="10" t="n"/>
+      <c r="AD101" s="10" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="10" t="n"/>
@@ -2312,6 +2624,12 @@
       <c r="V102" s="10" t="n"/>
       <c r="W102" s="10" t="n"/>
       <c r="X102" s="10" t="n"/>
+      <c r="Y102" s="10" t="n"/>
+      <c r="Z102" s="10" t="n"/>
+      <c r="AA102" s="10" t="n"/>
+      <c r="AB102" s="10" t="n"/>
+      <c r="AC102" s="10" t="n"/>
+      <c r="AD102" s="10" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="10" t="n"/>
@@ -2338,6 +2656,12 @@
       <c r="V103" s="10" t="n"/>
       <c r="W103" s="10" t="n"/>
       <c r="X103" s="10" t="n"/>
+      <c r="Y103" s="10" t="n"/>
+      <c r="Z103" s="10" t="n"/>
+      <c r="AA103" s="10" t="n"/>
+      <c r="AB103" s="10" t="n"/>
+      <c r="AC103" s="10" t="n"/>
+      <c r="AD103" s="10" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="10" t="n"/>
@@ -2364,6 +2688,12 @@
       <c r="V104" s="10" t="n"/>
       <c r="W104" s="10" t="n"/>
       <c r="X104" s="10" t="n"/>
+      <c r="Y104" s="10" t="n"/>
+      <c r="Z104" s="10" t="n"/>
+      <c r="AA104" s="10" t="n"/>
+      <c r="AB104" s="10" t="n"/>
+      <c r="AC104" s="10" t="n"/>
+      <c r="AD104" s="10" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="10" t="n"/>
@@ -2390,6 +2720,12 @@
       <c r="V105" s="10" t="n"/>
       <c r="W105" s="10" t="n"/>
       <c r="X105" s="10" t="n"/>
+      <c r="Y105" s="10" t="n"/>
+      <c r="Z105" s="10" t="n"/>
+      <c r="AA105" s="10" t="n"/>
+      <c r="AB105" s="10" t="n"/>
+      <c r="AC105" s="10" t="n"/>
+      <c r="AD105" s="10" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="10" t="n"/>
@@ -2416,6 +2752,12 @@
       <c r="V106" s="10" t="n"/>
       <c r="W106" s="10" t="n"/>
       <c r="X106" s="10" t="n"/>
+      <c r="Y106" s="10" t="n"/>
+      <c r="Z106" s="10" t="n"/>
+      <c r="AA106" s="10" t="n"/>
+      <c r="AB106" s="10" t="n"/>
+      <c r="AC106" s="10" t="n"/>
+      <c r="AD106" s="10" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="10" t="n"/>
@@ -2442,6 +2784,12 @@
       <c r="V107" s="10" t="n"/>
       <c r="W107" s="10" t="n"/>
       <c r="X107" s="10" t="n"/>
+      <c r="Y107" s="10" t="n"/>
+      <c r="Z107" s="10" t="n"/>
+      <c r="AA107" s="10" t="n"/>
+      <c r="AB107" s="10" t="n"/>
+      <c r="AC107" s="10" t="n"/>
+      <c r="AD107" s="10" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="10" t="n"/>
@@ -2468,6 +2816,12 @@
       <c r="V108" s="10" t="n"/>
       <c r="W108" s="10" t="n"/>
       <c r="X108" s="10" t="n"/>
+      <c r="Y108" s="10" t="n"/>
+      <c r="Z108" s="10" t="n"/>
+      <c r="AA108" s="10" t="n"/>
+      <c r="AB108" s="10" t="n"/>
+      <c r="AC108" s="10" t="n"/>
+      <c r="AD108" s="10" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="10" t="n"/>
@@ -2494,6 +2848,12 @@
       <c r="V109" s="10" t="n"/>
       <c r="W109" s="10" t="n"/>
       <c r="X109" s="10" t="n"/>
+      <c r="Y109" s="10" t="n"/>
+      <c r="Z109" s="10" t="n"/>
+      <c r="AA109" s="10" t="n"/>
+      <c r="AB109" s="10" t="n"/>
+      <c r="AC109" s="10" t="n"/>
+      <c r="AD109" s="10" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="10" t="n"/>
@@ -2520,6 +2880,12 @@
       <c r="V110" s="10" t="n"/>
       <c r="W110" s="10" t="n"/>
       <c r="X110" s="10" t="n"/>
+      <c r="Y110" s="10" t="n"/>
+      <c r="Z110" s="10" t="n"/>
+      <c r="AA110" s="10" t="n"/>
+      <c r="AB110" s="10" t="n"/>
+      <c r="AC110" s="10" t="n"/>
+      <c r="AD110" s="10" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="10" t="n"/>
@@ -2546,6 +2912,12 @@
       <c r="V111" s="10" t="n"/>
       <c r="W111" s="10" t="n"/>
       <c r="X111" s="10" t="n"/>
+      <c r="Y111" s="10" t="n"/>
+      <c r="Z111" s="10" t="n"/>
+      <c r="AA111" s="10" t="n"/>
+      <c r="AB111" s="10" t="n"/>
+      <c r="AC111" s="10" t="n"/>
+      <c r="AD111" s="10" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="10" t="n"/>
@@ -2572,6 +2944,12 @@
       <c r="V112" s="10" t="n"/>
       <c r="W112" s="10" t="n"/>
       <c r="X112" s="10" t="n"/>
+      <c r="Y112" s="10" t="n"/>
+      <c r="Z112" s="10" t="n"/>
+      <c r="AA112" s="10" t="n"/>
+      <c r="AB112" s="10" t="n"/>
+      <c r="AC112" s="10" t="n"/>
+      <c r="AD112" s="10" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="10" t="n"/>
@@ -2598,6 +2976,12 @@
       <c r="V113" s="10" t="n"/>
       <c r="W113" s="10" t="n"/>
       <c r="X113" s="10" t="n"/>
+      <c r="Y113" s="10" t="n"/>
+      <c r="Z113" s="10" t="n"/>
+      <c r="AA113" s="10" t="n"/>
+      <c r="AB113" s="10" t="n"/>
+      <c r="AC113" s="10" t="n"/>
+      <c r="AD113" s="10" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="10" t="n"/>
@@ -2624,6 +3008,12 @@
       <c r="V114" s="10" t="n"/>
       <c r="W114" s="10" t="n"/>
       <c r="X114" s="10" t="n"/>
+      <c r="Y114" s="10" t="n"/>
+      <c r="Z114" s="10" t="n"/>
+      <c r="AA114" s="10" t="n"/>
+      <c r="AB114" s="10" t="n"/>
+      <c r="AC114" s="10" t="n"/>
+      <c r="AD114" s="10" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="10" t="n"/>
@@ -2650,6 +3040,12 @@
       <c r="V115" s="10" t="n"/>
       <c r="W115" s="10" t="n"/>
       <c r="X115" s="10" t="n"/>
+      <c r="Y115" s="10" t="n"/>
+      <c r="Z115" s="10" t="n"/>
+      <c r="AA115" s="10" t="n"/>
+      <c r="AB115" s="10" t="n"/>
+      <c r="AC115" s="10" t="n"/>
+      <c r="AD115" s="10" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="10" t="n"/>
@@ -2676,6 +3072,12 @@
       <c r="V116" s="10" t="n"/>
       <c r="W116" s="10" t="n"/>
       <c r="X116" s="10" t="n"/>
+      <c r="Y116" s="10" t="n"/>
+      <c r="Z116" s="10" t="n"/>
+      <c r="AA116" s="10" t="n"/>
+      <c r="AB116" s="10" t="n"/>
+      <c r="AC116" s="10" t="n"/>
+      <c r="AD116" s="10" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="10" t="n"/>
@@ -2702,6 +3104,12 @@
       <c r="V117" s="10" t="n"/>
       <c r="W117" s="10" t="n"/>
       <c r="X117" s="10" t="n"/>
+      <c r="Y117" s="10" t="n"/>
+      <c r="Z117" s="10" t="n"/>
+      <c r="AA117" s="10" t="n"/>
+      <c r="AB117" s="10" t="n"/>
+      <c r="AC117" s="10" t="n"/>
+      <c r="AD117" s="10" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="10" t="n"/>
@@ -2728,6 +3136,12 @@
       <c r="V118" s="10" t="n"/>
       <c r="W118" s="10" t="n"/>
       <c r="X118" s="10" t="n"/>
+      <c r="Y118" s="10" t="n"/>
+      <c r="Z118" s="10" t="n"/>
+      <c r="AA118" s="10" t="n"/>
+      <c r="AB118" s="10" t="n"/>
+      <c r="AC118" s="10" t="n"/>
+      <c r="AD118" s="10" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="10" t="n"/>
@@ -2754,6 +3168,12 @@
       <c r="V119" s="10" t="n"/>
       <c r="W119" s="10" t="n"/>
       <c r="X119" s="10" t="n"/>
+      <c r="Y119" s="10" t="n"/>
+      <c r="Z119" s="10" t="n"/>
+      <c r="AA119" s="10" t="n"/>
+      <c r="AB119" s="10" t="n"/>
+      <c r="AC119" s="10" t="n"/>
+      <c r="AD119" s="10" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="10" t="n"/>
@@ -2780,6 +3200,12 @@
       <c r="V120" s="10" t="n"/>
       <c r="W120" s="10" t="n"/>
       <c r="X120" s="10" t="n"/>
+      <c r="Y120" s="10" t="n"/>
+      <c r="Z120" s="10" t="n"/>
+      <c r="AA120" s="10" t="n"/>
+      <c r="AB120" s="10" t="n"/>
+      <c r="AC120" s="10" t="n"/>
+      <c r="AD120" s="10" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="10" t="n"/>
@@ -2806,6 +3232,12 @@
       <c r="V121" s="10" t="n"/>
       <c r="W121" s="10" t="n"/>
       <c r="X121" s="10" t="n"/>
+      <c r="Y121" s="10" t="n"/>
+      <c r="Z121" s="10" t="n"/>
+      <c r="AA121" s="10" t="n"/>
+      <c r="AB121" s="10" t="n"/>
+      <c r="AC121" s="10" t="n"/>
+      <c r="AD121" s="10" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="10" t="n"/>
@@ -2832,6 +3264,12 @@
       <c r="V122" s="10" t="n"/>
       <c r="W122" s="10" t="n"/>
       <c r="X122" s="10" t="n"/>
+      <c r="Y122" s="10" t="n"/>
+      <c r="Z122" s="10" t="n"/>
+      <c r="AA122" s="10" t="n"/>
+      <c r="AB122" s="10" t="n"/>
+      <c r="AC122" s="10" t="n"/>
+      <c r="AD122" s="10" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="10" t="n"/>
@@ -2858,6 +3296,12 @@
       <c r="V123" s="10" t="n"/>
       <c r="W123" s="10" t="n"/>
       <c r="X123" s="10" t="n"/>
+      <c r="Y123" s="10" t="n"/>
+      <c r="Z123" s="10" t="n"/>
+      <c r="AA123" s="10" t="n"/>
+      <c r="AB123" s="10" t="n"/>
+      <c r="AC123" s="10" t="n"/>
+      <c r="AD123" s="10" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="10" t="n"/>
@@ -2884,6 +3328,12 @@
       <c r="V124" s="10" t="n"/>
       <c r="W124" s="10" t="n"/>
       <c r="X124" s="10" t="n"/>
+      <c r="Y124" s="10" t="n"/>
+      <c r="Z124" s="10" t="n"/>
+      <c r="AA124" s="10" t="n"/>
+      <c r="AB124" s="10" t="n"/>
+      <c r="AC124" s="10" t="n"/>
+      <c r="AD124" s="10" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="10" t="n"/>
@@ -2910,6 +3360,12 @@
       <c r="V125" s="10" t="n"/>
       <c r="W125" s="10" t="n"/>
       <c r="X125" s="10" t="n"/>
+      <c r="Y125" s="10" t="n"/>
+      <c r="Z125" s="10" t="n"/>
+      <c r="AA125" s="10" t="n"/>
+      <c r="AB125" s="10" t="n"/>
+      <c r="AC125" s="10" t="n"/>
+      <c r="AD125" s="10" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="10" t="n"/>
@@ -2936,6 +3392,12 @@
       <c r="V126" s="10" t="n"/>
       <c r="W126" s="10" t="n"/>
       <c r="X126" s="10" t="n"/>
+      <c r="Y126" s="10" t="n"/>
+      <c r="Z126" s="10" t="n"/>
+      <c r="AA126" s="10" t="n"/>
+      <c r="AB126" s="10" t="n"/>
+      <c r="AC126" s="10" t="n"/>
+      <c r="AD126" s="10" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="10" t="n"/>
@@ -2962,6 +3424,12 @@
       <c r="V127" s="10" t="n"/>
       <c r="W127" s="10" t="n"/>
       <c r="X127" s="10" t="n"/>
+      <c r="Y127" s="10" t="n"/>
+      <c r="Z127" s="10" t="n"/>
+      <c r="AA127" s="10" t="n"/>
+      <c r="AB127" s="10" t="n"/>
+      <c r="AC127" s="10" t="n"/>
+      <c r="AD127" s="10" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="10" t="n"/>
@@ -2988,6 +3456,12 @@
       <c r="V128" s="10" t="n"/>
       <c r="W128" s="10" t="n"/>
       <c r="X128" s="10" t="n"/>
+      <c r="Y128" s="10" t="n"/>
+      <c r="Z128" s="10" t="n"/>
+      <c r="AA128" s="10" t="n"/>
+      <c r="AB128" s="10" t="n"/>
+      <c r="AC128" s="10" t="n"/>
+      <c r="AD128" s="10" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="10" t="n"/>
@@ -3014,6 +3488,12 @@
       <c r="V129" s="10" t="n"/>
       <c r="W129" s="10" t="n"/>
       <c r="X129" s="10" t="n"/>
+      <c r="Y129" s="10" t="n"/>
+      <c r="Z129" s="10" t="n"/>
+      <c r="AA129" s="10" t="n"/>
+      <c r="AB129" s="10" t="n"/>
+      <c r="AC129" s="10" t="n"/>
+      <c r="AD129" s="10" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="10" t="n"/>
@@ -3040,6 +3520,12 @@
       <c r="V130" s="10" t="n"/>
       <c r="W130" s="10" t="n"/>
       <c r="X130" s="10" t="n"/>
+      <c r="Y130" s="10" t="n"/>
+      <c r="Z130" s="10" t="n"/>
+      <c r="AA130" s="10" t="n"/>
+      <c r="AB130" s="10" t="n"/>
+      <c r="AC130" s="10" t="n"/>
+      <c r="AD130" s="10" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="10" t="n"/>
@@ -3066,6 +3552,12 @@
       <c r="V131" s="10" t="n"/>
       <c r="W131" s="10" t="n"/>
       <c r="X131" s="10" t="n"/>
+      <c r="Y131" s="10" t="n"/>
+      <c r="Z131" s="10" t="n"/>
+      <c r="AA131" s="10" t="n"/>
+      <c r="AB131" s="10" t="n"/>
+      <c r="AC131" s="10" t="n"/>
+      <c r="AD131" s="10" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="10" t="n"/>
@@ -3092,6 +3584,12 @@
       <c r="V132" s="10" t="n"/>
       <c r="W132" s="10" t="n"/>
       <c r="X132" s="10" t="n"/>
+      <c r="Y132" s="10" t="n"/>
+      <c r="Z132" s="10" t="n"/>
+      <c r="AA132" s="10" t="n"/>
+      <c r="AB132" s="10" t="n"/>
+      <c r="AC132" s="10" t="n"/>
+      <c r="AD132" s="10" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="10" t="n"/>
@@ -3118,6 +3616,12 @@
       <c r="V133" s="10" t="n"/>
       <c r="W133" s="10" t="n"/>
       <c r="X133" s="10" t="n"/>
+      <c r="Y133" s="10" t="n"/>
+      <c r="Z133" s="10" t="n"/>
+      <c r="AA133" s="10" t="n"/>
+      <c r="AB133" s="10" t="n"/>
+      <c r="AC133" s="10" t="n"/>
+      <c r="AD133" s="10" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="10" t="n"/>
@@ -3144,6 +3648,12 @@
       <c r="V134" s="10" t="n"/>
       <c r="W134" s="10" t="n"/>
       <c r="X134" s="10" t="n"/>
+      <c r="Y134" s="10" t="n"/>
+      <c r="Z134" s="10" t="n"/>
+      <c r="AA134" s="10" t="n"/>
+      <c r="AB134" s="10" t="n"/>
+      <c r="AC134" s="10" t="n"/>
+      <c r="AD134" s="10" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="10" t="n"/>
@@ -3170,6 +3680,12 @@
       <c r="V135" s="10" t="n"/>
       <c r="W135" s="10" t="n"/>
       <c r="X135" s="10" t="n"/>
+      <c r="Y135" s="10" t="n"/>
+      <c r="Z135" s="10" t="n"/>
+      <c r="AA135" s="10" t="n"/>
+      <c r="AB135" s="10" t="n"/>
+      <c r="AC135" s="10" t="n"/>
+      <c r="AD135" s="10" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="10" t="n"/>
@@ -3196,6 +3712,12 @@
       <c r="V136" s="10" t="n"/>
       <c r="W136" s="10" t="n"/>
       <c r="X136" s="10" t="n"/>
+      <c r="Y136" s="10" t="n"/>
+      <c r="Z136" s="10" t="n"/>
+      <c r="AA136" s="10" t="n"/>
+      <c r="AB136" s="10" t="n"/>
+      <c r="AC136" s="10" t="n"/>
+      <c r="AD136" s="10" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="10" t="n"/>
@@ -3222,6 +3744,12 @@
       <c r="V137" s="10" t="n"/>
       <c r="W137" s="10" t="n"/>
       <c r="X137" s="10" t="n"/>
+      <c r="Y137" s="10" t="n"/>
+      <c r="Z137" s="10" t="n"/>
+      <c r="AA137" s="10" t="n"/>
+      <c r="AB137" s="10" t="n"/>
+      <c r="AC137" s="10" t="n"/>
+      <c r="AD137" s="10" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="10" t="n"/>
@@ -3248,6 +3776,12 @@
       <c r="V138" s="10" t="n"/>
       <c r="W138" s="10" t="n"/>
       <c r="X138" s="10" t="n"/>
+      <c r="Y138" s="10" t="n"/>
+      <c r="Z138" s="10" t="n"/>
+      <c r="AA138" s="10" t="n"/>
+      <c r="AB138" s="10" t="n"/>
+      <c r="AC138" s="10" t="n"/>
+      <c r="AD138" s="10" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="10" t="n"/>
@@ -3274,6 +3808,12 @@
       <c r="V139" s="10" t="n"/>
       <c r="W139" s="10" t="n"/>
       <c r="X139" s="10" t="n"/>
+      <c r="Y139" s="10" t="n"/>
+      <c r="Z139" s="10" t="n"/>
+      <c r="AA139" s="10" t="n"/>
+      <c r="AB139" s="10" t="n"/>
+      <c r="AC139" s="10" t="n"/>
+      <c r="AD139" s="10" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="10" t="n"/>
@@ -3300,6 +3840,12 @@
       <c r="V140" s="10" t="n"/>
       <c r="W140" s="10" t="n"/>
       <c r="X140" s="10" t="n"/>
+      <c r="Y140" s="10" t="n"/>
+      <c r="Z140" s="10" t="n"/>
+      <c r="AA140" s="10" t="n"/>
+      <c r="AB140" s="10" t="n"/>
+      <c r="AC140" s="10" t="n"/>
+      <c r="AD140" s="10" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="10" t="n"/>
@@ -3326,6 +3872,12 @@
       <c r="V141" s="10" t="n"/>
       <c r="W141" s="10" t="n"/>
       <c r="X141" s="10" t="n"/>
+      <c r="Y141" s="10" t="n"/>
+      <c r="Z141" s="10" t="n"/>
+      <c r="AA141" s="10" t="n"/>
+      <c r="AB141" s="10" t="n"/>
+      <c r="AC141" s="10" t="n"/>
+      <c r="AD141" s="10" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="10" t="n"/>
@@ -3352,6 +3904,12 @@
       <c r="V142" s="10" t="n"/>
       <c r="W142" s="10" t="n"/>
       <c r="X142" s="10" t="n"/>
+      <c r="Y142" s="10" t="n"/>
+      <c r="Z142" s="10" t="n"/>
+      <c r="AA142" s="10" t="n"/>
+      <c r="AB142" s="10" t="n"/>
+      <c r="AC142" s="10" t="n"/>
+      <c r="AD142" s="10" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="10" t="n"/>
@@ -3378,6 +3936,12 @@
       <c r="V143" s="10" t="n"/>
       <c r="W143" s="10" t="n"/>
       <c r="X143" s="10" t="n"/>
+      <c r="Y143" s="10" t="n"/>
+      <c r="Z143" s="10" t="n"/>
+      <c r="AA143" s="10" t="n"/>
+      <c r="AB143" s="10" t="n"/>
+      <c r="AC143" s="10" t="n"/>
+      <c r="AD143" s="10" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="10" t="n"/>
@@ -3404,6 +3968,12 @@
       <c r="V144" s="10" t="n"/>
       <c r="W144" s="10" t="n"/>
       <c r="X144" s="10" t="n"/>
+      <c r="Y144" s="10" t="n"/>
+      <c r="Z144" s="10" t="n"/>
+      <c r="AA144" s="10" t="n"/>
+      <c r="AB144" s="10" t="n"/>
+      <c r="AC144" s="10" t="n"/>
+      <c r="AD144" s="10" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="10" t="n"/>
@@ -3430,6 +4000,12 @@
       <c r="V145" s="10" t="n"/>
       <c r="W145" s="10" t="n"/>
       <c r="X145" s="10" t="n"/>
+      <c r="Y145" s="10" t="n"/>
+      <c r="Z145" s="10" t="n"/>
+      <c r="AA145" s="10" t="n"/>
+      <c r="AB145" s="10" t="n"/>
+      <c r="AC145" s="10" t="n"/>
+      <c r="AD145" s="10" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="10" t="n"/>
@@ -3456,6 +4032,12 @@
       <c r="V146" s="10" t="n"/>
       <c r="W146" s="10" t="n"/>
       <c r="X146" s="10" t="n"/>
+      <c r="Y146" s="10" t="n"/>
+      <c r="Z146" s="10" t="n"/>
+      <c r="AA146" s="10" t="n"/>
+      <c r="AB146" s="10" t="n"/>
+      <c r="AC146" s="10" t="n"/>
+      <c r="AD146" s="10" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="10" t="n"/>
@@ -3482,6 +4064,12 @@
       <c r="V147" s="10" t="n"/>
       <c r="W147" s="10" t="n"/>
       <c r="X147" s="10" t="n"/>
+      <c r="Y147" s="10" t="n"/>
+      <c r="Z147" s="10" t="n"/>
+      <c r="AA147" s="10" t="n"/>
+      <c r="AB147" s="10" t="n"/>
+      <c r="AC147" s="10" t="n"/>
+      <c r="AD147" s="10" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="10" t="n"/>
@@ -3508,6 +4096,12 @@
       <c r="V148" s="10" t="n"/>
       <c r="W148" s="10" t="n"/>
       <c r="X148" s="10" t="n"/>
+      <c r="Y148" s="10" t="n"/>
+      <c r="Z148" s="10" t="n"/>
+      <c r="AA148" s="10" t="n"/>
+      <c r="AB148" s="10" t="n"/>
+      <c r="AC148" s="10" t="n"/>
+      <c r="AD148" s="10" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="10" t="n"/>
@@ -3534,6 +4128,12 @@
       <c r="V149" s="10" t="n"/>
       <c r="W149" s="10" t="n"/>
       <c r="X149" s="10" t="n"/>
+      <c r="Y149" s="10" t="n"/>
+      <c r="Z149" s="10" t="n"/>
+      <c r="AA149" s="10" t="n"/>
+      <c r="AB149" s="10" t="n"/>
+      <c r="AC149" s="10" t="n"/>
+      <c r="AD149" s="10" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="10" t="n"/>
@@ -3560,6 +4160,12 @@
       <c r="V150" s="10" t="n"/>
       <c r="W150" s="10" t="n"/>
       <c r="X150" s="10" t="n"/>
+      <c r="Y150" s="10" t="n"/>
+      <c r="Z150" s="10" t="n"/>
+      <c r="AA150" s="10" t="n"/>
+      <c r="AB150" s="10" t="n"/>
+      <c r="AC150" s="10" t="n"/>
+      <c r="AD150" s="10" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="10" t="n"/>
@@ -3586,6 +4192,12 @@
       <c r="V151" s="10" t="n"/>
       <c r="W151" s="10" t="n"/>
       <c r="X151" s="10" t="n"/>
+      <c r="Y151" s="10" t="n"/>
+      <c r="Z151" s="10" t="n"/>
+      <c r="AA151" s="10" t="n"/>
+      <c r="AB151" s="10" t="n"/>
+      <c r="AC151" s="10" t="n"/>
+      <c r="AD151" s="10" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="10" t="n"/>
@@ -3612,6 +4224,12 @@
       <c r="V152" s="10" t="n"/>
       <c r="W152" s="10" t="n"/>
       <c r="X152" s="10" t="n"/>
+      <c r="Y152" s="10" t="n"/>
+      <c r="Z152" s="10" t="n"/>
+      <c r="AA152" s="10" t="n"/>
+      <c r="AB152" s="10" t="n"/>
+      <c r="AC152" s="10" t="n"/>
+      <c r="AD152" s="10" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="10" t="n"/>
@@ -3638,6 +4256,12 @@
       <c r="V153" s="10" t="n"/>
       <c r="W153" s="10" t="n"/>
       <c r="X153" s="10" t="n"/>
+      <c r="Y153" s="10" t="n"/>
+      <c r="Z153" s="10" t="n"/>
+      <c r="AA153" s="10" t="n"/>
+      <c r="AB153" s="10" t="n"/>
+      <c r="AC153" s="10" t="n"/>
+      <c r="AD153" s="10" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="10" t="n"/>
@@ -3664,6 +4288,12 @@
       <c r="V154" s="10" t="n"/>
       <c r="W154" s="10" t="n"/>
       <c r="X154" s="10" t="n"/>
+      <c r="Y154" s="10" t="n"/>
+      <c r="Z154" s="10" t="n"/>
+      <c r="AA154" s="10" t="n"/>
+      <c r="AB154" s="10" t="n"/>
+      <c r="AC154" s="10" t="n"/>
+      <c r="AD154" s="10" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="10" t="n"/>
@@ -3690,6 +4320,12 @@
       <c r="V155" s="10" t="n"/>
       <c r="W155" s="10" t="n"/>
       <c r="X155" s="10" t="n"/>
+      <c r="Y155" s="10" t="n"/>
+      <c r="Z155" s="10" t="n"/>
+      <c r="AA155" s="10" t="n"/>
+      <c r="AB155" s="10" t="n"/>
+      <c r="AC155" s="10" t="n"/>
+      <c r="AD155" s="10" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="10" t="n"/>
@@ -3716,6 +4352,12 @@
       <c r="V156" s="10" t="n"/>
       <c r="W156" s="10" t="n"/>
       <c r="X156" s="10" t="n"/>
+      <c r="Y156" s="10" t="n"/>
+      <c r="Z156" s="10" t="n"/>
+      <c r="AA156" s="10" t="n"/>
+      <c r="AB156" s="10" t="n"/>
+      <c r="AC156" s="10" t="n"/>
+      <c r="AD156" s="10" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="10" t="n"/>
@@ -3742,6 +4384,12 @@
       <c r="V157" s="10" t="n"/>
       <c r="W157" s="10" t="n"/>
       <c r="X157" s="10" t="n"/>
+      <c r="Y157" s="10" t="n"/>
+      <c r="Z157" s="10" t="n"/>
+      <c r="AA157" s="10" t="n"/>
+      <c r="AB157" s="10" t="n"/>
+      <c r="AC157" s="10" t="n"/>
+      <c r="AD157" s="10" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="10" t="n"/>
@@ -3768,6 +4416,12 @@
       <c r="V158" s="10" t="n"/>
       <c r="W158" s="10" t="n"/>
       <c r="X158" s="10" t="n"/>
+      <c r="Y158" s="10" t="n"/>
+      <c r="Z158" s="10" t="n"/>
+      <c r="AA158" s="10" t="n"/>
+      <c r="AB158" s="10" t="n"/>
+      <c r="AC158" s="10" t="n"/>
+      <c r="AD158" s="10" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="10" t="n"/>
@@ -3794,6 +4448,12 @@
       <c r="V159" s="10" t="n"/>
       <c r="W159" s="10" t="n"/>
       <c r="X159" s="10" t="n"/>
+      <c r="Y159" s="10" t="n"/>
+      <c r="Z159" s="10" t="n"/>
+      <c r="AA159" s="10" t="n"/>
+      <c r="AB159" s="10" t="n"/>
+      <c r="AC159" s="10" t="n"/>
+      <c r="AD159" s="10" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="10" t="n"/>
@@ -3820,6 +4480,12 @@
       <c r="V160" s="10" t="n"/>
       <c r="W160" s="10" t="n"/>
       <c r="X160" s="10" t="n"/>
+      <c r="Y160" s="10" t="n"/>
+      <c r="Z160" s="10" t="n"/>
+      <c r="AA160" s="10" t="n"/>
+      <c r="AB160" s="10" t="n"/>
+      <c r="AC160" s="10" t="n"/>
+      <c r="AD160" s="10" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="10" t="n"/>
@@ -3846,6 +4512,12 @@
       <c r="V161" s="10" t="n"/>
       <c r="W161" s="10" t="n"/>
       <c r="X161" s="10" t="n"/>
+      <c r="Y161" s="10" t="n"/>
+      <c r="Z161" s="10" t="n"/>
+      <c r="AA161" s="10" t="n"/>
+      <c r="AB161" s="10" t="n"/>
+      <c r="AC161" s="10" t="n"/>
+      <c r="AD161" s="10" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="10" t="n"/>
@@ -3872,6 +4544,12 @@
       <c r="V162" s="10" t="n"/>
       <c r="W162" s="10" t="n"/>
       <c r="X162" s="10" t="n"/>
+      <c r="Y162" s="10" t="n"/>
+      <c r="Z162" s="10" t="n"/>
+      <c r="AA162" s="10" t="n"/>
+      <c r="AB162" s="10" t="n"/>
+      <c r="AC162" s="10" t="n"/>
+      <c r="AD162" s="10" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="10" t="n"/>
@@ -3898,6 +4576,12 @@
       <c r="V163" s="10" t="n"/>
       <c r="W163" s="10" t="n"/>
       <c r="X163" s="10" t="n"/>
+      <c r="Y163" s="10" t="n"/>
+      <c r="Z163" s="10" t="n"/>
+      <c r="AA163" s="10" t="n"/>
+      <c r="AB163" s="10" t="n"/>
+      <c r="AC163" s="10" t="n"/>
+      <c r="AD163" s="10" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="10" t="n"/>
@@ -3924,6 +4608,12 @@
       <c r="V164" s="10" t="n"/>
       <c r="W164" s="10" t="n"/>
       <c r="X164" s="10" t="n"/>
+      <c r="Y164" s="10" t="n"/>
+      <c r="Z164" s="10" t="n"/>
+      <c r="AA164" s="10" t="n"/>
+      <c r="AB164" s="10" t="n"/>
+      <c r="AC164" s="10" t="n"/>
+      <c r="AD164" s="10" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="10" t="n"/>
@@ -3950,6 +4640,12 @@
       <c r="V165" s="10" t="n"/>
       <c r="W165" s="10" t="n"/>
       <c r="X165" s="10" t="n"/>
+      <c r="Y165" s="10" t="n"/>
+      <c r="Z165" s="10" t="n"/>
+      <c r="AA165" s="10" t="n"/>
+      <c r="AB165" s="10" t="n"/>
+      <c r="AC165" s="10" t="n"/>
+      <c r="AD165" s="10" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="10" t="n"/>
@@ -3976,6 +4672,12 @@
       <c r="V166" s="10" t="n"/>
       <c r="W166" s="10" t="n"/>
       <c r="X166" s="10" t="n"/>
+      <c r="Y166" s="10" t="n"/>
+      <c r="Z166" s="10" t="n"/>
+      <c r="AA166" s="10" t="n"/>
+      <c r="AB166" s="10" t="n"/>
+      <c r="AC166" s="10" t="n"/>
+      <c r="AD166" s="10" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="10" t="n"/>
@@ -4002,6 +4704,12 @@
       <c r="V167" s="10" t="n"/>
       <c r="W167" s="10" t="n"/>
       <c r="X167" s="10" t="n"/>
+      <c r="Y167" s="10" t="n"/>
+      <c r="Z167" s="10" t="n"/>
+      <c r="AA167" s="10" t="n"/>
+      <c r="AB167" s="10" t="n"/>
+      <c r="AC167" s="10" t="n"/>
+      <c r="AD167" s="10" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="10" t="n"/>
@@ -4028,6 +4736,12 @@
       <c r="V168" s="10" t="n"/>
       <c r="W168" s="10" t="n"/>
       <c r="X168" s="10" t="n"/>
+      <c r="Y168" s="10" t="n"/>
+      <c r="Z168" s="10" t="n"/>
+      <c r="AA168" s="10" t="n"/>
+      <c r="AB168" s="10" t="n"/>
+      <c r="AC168" s="10" t="n"/>
+      <c r="AD168" s="10" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="10" t="n"/>
@@ -4054,6 +4768,12 @@
       <c r="V169" s="10" t="n"/>
       <c r="W169" s="10" t="n"/>
       <c r="X169" s="10" t="n"/>
+      <c r="Y169" s="10" t="n"/>
+      <c r="Z169" s="10" t="n"/>
+      <c r="AA169" s="10" t="n"/>
+      <c r="AB169" s="10" t="n"/>
+      <c r="AC169" s="10" t="n"/>
+      <c r="AD169" s="10" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="10" t="n"/>
@@ -4080,6 +4800,12 @@
       <c r="V170" s="10" t="n"/>
       <c r="W170" s="10" t="n"/>
       <c r="X170" s="10" t="n"/>
+      <c r="Y170" s="10" t="n"/>
+      <c r="Z170" s="10" t="n"/>
+      <c r="AA170" s="10" t="n"/>
+      <c r="AB170" s="10" t="n"/>
+      <c r="AC170" s="10" t="n"/>
+      <c r="AD170" s="10" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="10" t="n"/>
@@ -4106,6 +4832,12 @@
       <c r="V171" s="10" t="n"/>
       <c r="W171" s="10" t="n"/>
       <c r="X171" s="10" t="n"/>
+      <c r="Y171" s="10" t="n"/>
+      <c r="Z171" s="10" t="n"/>
+      <c r="AA171" s="10" t="n"/>
+      <c r="AB171" s="10" t="n"/>
+      <c r="AC171" s="10" t="n"/>
+      <c r="AD171" s="10" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="10" t="n"/>
@@ -4132,6 +4864,12 @@
       <c r="V172" s="10" t="n"/>
       <c r="W172" s="10" t="n"/>
       <c r="X172" s="10" t="n"/>
+      <c r="Y172" s="10" t="n"/>
+      <c r="Z172" s="10" t="n"/>
+      <c r="AA172" s="10" t="n"/>
+      <c r="AB172" s="10" t="n"/>
+      <c r="AC172" s="10" t="n"/>
+      <c r="AD172" s="10" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="10" t="n"/>
@@ -4158,6 +4896,12 @@
       <c r="V173" s="10" t="n"/>
       <c r="W173" s="10" t="n"/>
       <c r="X173" s="10" t="n"/>
+      <c r="Y173" s="10" t="n"/>
+      <c r="Z173" s="10" t="n"/>
+      <c r="AA173" s="10" t="n"/>
+      <c r="AB173" s="10" t="n"/>
+      <c r="AC173" s="10" t="n"/>
+      <c r="AD173" s="10" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="10" t="n"/>
@@ -4184,6 +4928,12 @@
       <c r="V174" s="10" t="n"/>
       <c r="W174" s="10" t="n"/>
       <c r="X174" s="10" t="n"/>
+      <c r="Y174" s="10" t="n"/>
+      <c r="Z174" s="10" t="n"/>
+      <c r="AA174" s="10" t="n"/>
+      <c r="AB174" s="10" t="n"/>
+      <c r="AC174" s="10" t="n"/>
+      <c r="AD174" s="10" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="10" t="n"/>
@@ -4210,6 +4960,12 @@
       <c r="V175" s="10" t="n"/>
       <c r="W175" s="10" t="n"/>
       <c r="X175" s="10" t="n"/>
+      <c r="Y175" s="10" t="n"/>
+      <c r="Z175" s="10" t="n"/>
+      <c r="AA175" s="10" t="n"/>
+      <c r="AB175" s="10" t="n"/>
+      <c r="AC175" s="10" t="n"/>
+      <c r="AD175" s="10" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="10" t="n"/>
@@ -4236,6 +4992,12 @@
       <c r="V176" s="10" t="n"/>
       <c r="W176" s="10" t="n"/>
       <c r="X176" s="10" t="n"/>
+      <c r="Y176" s="10" t="n"/>
+      <c r="Z176" s="10" t="n"/>
+      <c r="AA176" s="10" t="n"/>
+      <c r="AB176" s="10" t="n"/>
+      <c r="AC176" s="10" t="n"/>
+      <c r="AD176" s="10" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="10" t="n"/>
@@ -4262,6 +5024,12 @@
       <c r="V177" s="10" t="n"/>
       <c r="W177" s="10" t="n"/>
       <c r="X177" s="10" t="n"/>
+      <c r="Y177" s="10" t="n"/>
+      <c r="Z177" s="10" t="n"/>
+      <c r="AA177" s="10" t="n"/>
+      <c r="AB177" s="10" t="n"/>
+      <c r="AC177" s="10" t="n"/>
+      <c r="AD177" s="10" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="10" t="n"/>
@@ -4288,6 +5056,12 @@
       <c r="V178" s="10" t="n"/>
       <c r="W178" s="10" t="n"/>
       <c r="X178" s="10" t="n"/>
+      <c r="Y178" s="10" t="n"/>
+      <c r="Z178" s="10" t="n"/>
+      <c r="AA178" s="10" t="n"/>
+      <c r="AB178" s="10" t="n"/>
+      <c r="AC178" s="10" t="n"/>
+      <c r="AD178" s="10" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="10" t="n"/>
@@ -4314,6 +5088,12 @@
       <c r="V179" s="10" t="n"/>
       <c r="W179" s="10" t="n"/>
       <c r="X179" s="10" t="n"/>
+      <c r="Y179" s="10" t="n"/>
+      <c r="Z179" s="10" t="n"/>
+      <c r="AA179" s="10" t="n"/>
+      <c r="AB179" s="10" t="n"/>
+      <c r="AC179" s="10" t="n"/>
+      <c r="AD179" s="10" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="10" t="n"/>
@@ -4340,6 +5120,12 @@
       <c r="V180" s="10" t="n"/>
       <c r="W180" s="10" t="n"/>
       <c r="X180" s="10" t="n"/>
+      <c r="Y180" s="10" t="n"/>
+      <c r="Z180" s="10" t="n"/>
+      <c r="AA180" s="10" t="n"/>
+      <c r="AB180" s="10" t="n"/>
+      <c r="AC180" s="10" t="n"/>
+      <c r="AD180" s="10" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="10" t="n"/>
@@ -4366,6 +5152,12 @@
       <c r="V181" s="10" t="n"/>
       <c r="W181" s="10" t="n"/>
       <c r="X181" s="10" t="n"/>
+      <c r="Y181" s="10" t="n"/>
+      <c r="Z181" s="10" t="n"/>
+      <c r="AA181" s="10" t="n"/>
+      <c r="AB181" s="10" t="n"/>
+      <c r="AC181" s="10" t="n"/>
+      <c r="AD181" s="10" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="10" t="n"/>
@@ -4392,6 +5184,12 @@
       <c r="V182" s="10" t="n"/>
       <c r="W182" s="10" t="n"/>
       <c r="X182" s="10" t="n"/>
+      <c r="Y182" s="10" t="n"/>
+      <c r="Z182" s="10" t="n"/>
+      <c r="AA182" s="10" t="n"/>
+      <c r="AB182" s="10" t="n"/>
+      <c r="AC182" s="10" t="n"/>
+      <c r="AD182" s="10" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="10" t="n"/>
@@ -4418,6 +5216,12 @@
       <c r="V183" s="10" t="n"/>
       <c r="W183" s="10" t="n"/>
       <c r="X183" s="10" t="n"/>
+      <c r="Y183" s="10" t="n"/>
+      <c r="Z183" s="10" t="n"/>
+      <c r="AA183" s="10" t="n"/>
+      <c r="AB183" s="10" t="n"/>
+      <c r="AC183" s="10" t="n"/>
+      <c r="AD183" s="10" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="10" t="n"/>
@@ -4444,6 +5248,12 @@
       <c r="V184" s="10" t="n"/>
       <c r="W184" s="10" t="n"/>
       <c r="X184" s="10" t="n"/>
+      <c r="Y184" s="10" t="n"/>
+      <c r="Z184" s="10" t="n"/>
+      <c r="AA184" s="10" t="n"/>
+      <c r="AB184" s="10" t="n"/>
+      <c r="AC184" s="10" t="n"/>
+      <c r="AD184" s="10" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="10" t="n"/>
@@ -4470,6 +5280,12 @@
       <c r="V185" s="10" t="n"/>
       <c r="W185" s="10" t="n"/>
       <c r="X185" s="10" t="n"/>
+      <c r="Y185" s="10" t="n"/>
+      <c r="Z185" s="10" t="n"/>
+      <c r="AA185" s="10" t="n"/>
+      <c r="AB185" s="10" t="n"/>
+      <c r="AC185" s="10" t="n"/>
+      <c r="AD185" s="10" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="10" t="n"/>
@@ -4496,6 +5312,12 @@
       <c r="V186" s="10" t="n"/>
       <c r="W186" s="10" t="n"/>
       <c r="X186" s="10" t="n"/>
+      <c r="Y186" s="10" t="n"/>
+      <c r="Z186" s="10" t="n"/>
+      <c r="AA186" s="10" t="n"/>
+      <c r="AB186" s="10" t="n"/>
+      <c r="AC186" s="10" t="n"/>
+      <c r="AD186" s="10" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="10" t="n"/>
@@ -4522,6 +5344,12 @@
       <c r="V187" s="10" t="n"/>
       <c r="W187" s="10" t="n"/>
       <c r="X187" s="10" t="n"/>
+      <c r="Y187" s="10" t="n"/>
+      <c r="Z187" s="10" t="n"/>
+      <c r="AA187" s="10" t="n"/>
+      <c r="AB187" s="10" t="n"/>
+      <c r="AC187" s="10" t="n"/>
+      <c r="AD187" s="10" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="10" t="n"/>
@@ -4548,6 +5376,12 @@
       <c r="V188" s="10" t="n"/>
       <c r="W188" s="10" t="n"/>
       <c r="X188" s="10" t="n"/>
+      <c r="Y188" s="10" t="n"/>
+      <c r="Z188" s="10" t="n"/>
+      <c r="AA188" s="10" t="n"/>
+      <c r="AB188" s="10" t="n"/>
+      <c r="AC188" s="10" t="n"/>
+      <c r="AD188" s="10" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="10" t="n"/>
@@ -4574,6 +5408,12 @@
       <c r="V189" s="10" t="n"/>
       <c r="W189" s="10" t="n"/>
       <c r="X189" s="10" t="n"/>
+      <c r="Y189" s="10" t="n"/>
+      <c r="Z189" s="10" t="n"/>
+      <c r="AA189" s="10" t="n"/>
+      <c r="AB189" s="10" t="n"/>
+      <c r="AC189" s="10" t="n"/>
+      <c r="AD189" s="10" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="10" t="n"/>
@@ -4600,6 +5440,12 @@
       <c r="V190" s="10" t="n"/>
       <c r="W190" s="10" t="n"/>
       <c r="X190" s="10" t="n"/>
+      <c r="Y190" s="10" t="n"/>
+      <c r="Z190" s="10" t="n"/>
+      <c r="AA190" s="10" t="n"/>
+      <c r="AB190" s="10" t="n"/>
+      <c r="AC190" s="10" t="n"/>
+      <c r="AD190" s="10" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="10" t="n"/>
@@ -4626,6 +5472,12 @@
       <c r="V191" s="10" t="n"/>
       <c r="W191" s="10" t="n"/>
       <c r="X191" s="10" t="n"/>
+      <c r="Y191" s="10" t="n"/>
+      <c r="Z191" s="10" t="n"/>
+      <c r="AA191" s="10" t="n"/>
+      <c r="AB191" s="10" t="n"/>
+      <c r="AC191" s="10" t="n"/>
+      <c r="AD191" s="10" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="10" t="n"/>
@@ -4652,6 +5504,12 @@
       <c r="V192" s="10" t="n"/>
       <c r="W192" s="10" t="n"/>
       <c r="X192" s="10" t="n"/>
+      <c r="Y192" s="10" t="n"/>
+      <c r="Z192" s="10" t="n"/>
+      <c r="AA192" s="10" t="n"/>
+      <c r="AB192" s="10" t="n"/>
+      <c r="AC192" s="10" t="n"/>
+      <c r="AD192" s="10" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="10" t="n"/>
@@ -4678,6 +5536,12 @@
       <c r="V193" s="10" t="n"/>
       <c r="W193" s="10" t="n"/>
       <c r="X193" s="10" t="n"/>
+      <c r="Y193" s="10" t="n"/>
+      <c r="Z193" s="10" t="n"/>
+      <c r="AA193" s="10" t="n"/>
+      <c r="AB193" s="10" t="n"/>
+      <c r="AC193" s="10" t="n"/>
+      <c r="AD193" s="10" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="10" t="n"/>
@@ -4704,6 +5568,12 @@
       <c r="V194" s="10" t="n"/>
       <c r="W194" s="10" t="n"/>
       <c r="X194" s="10" t="n"/>
+      <c r="Y194" s="10" t="n"/>
+      <c r="Z194" s="10" t="n"/>
+      <c r="AA194" s="10" t="n"/>
+      <c r="AB194" s="10" t="n"/>
+      <c r="AC194" s="10" t="n"/>
+      <c r="AD194" s="10" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="10" t="n"/>
@@ -4730,6 +5600,12 @@
       <c r="V195" s="10" t="n"/>
       <c r="W195" s="10" t="n"/>
       <c r="X195" s="10" t="n"/>
+      <c r="Y195" s="10" t="n"/>
+      <c r="Z195" s="10" t="n"/>
+      <c r="AA195" s="10" t="n"/>
+      <c r="AB195" s="10" t="n"/>
+      <c r="AC195" s="10" t="n"/>
+      <c r="AD195" s="10" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="10" t="n"/>
@@ -4756,6 +5632,12 @@
       <c r="V196" s="10" t="n"/>
       <c r="W196" s="10" t="n"/>
       <c r="X196" s="10" t="n"/>
+      <c r="Y196" s="10" t="n"/>
+      <c r="Z196" s="10" t="n"/>
+      <c r="AA196" s="10" t="n"/>
+      <c r="AB196" s="10" t="n"/>
+      <c r="AC196" s="10" t="n"/>
+      <c r="AD196" s="10" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="10" t="n"/>
@@ -4782,6 +5664,12 @@
       <c r="V197" s="10" t="n"/>
       <c r="W197" s="10" t="n"/>
       <c r="X197" s="10" t="n"/>
+      <c r="Y197" s="10" t="n"/>
+      <c r="Z197" s="10" t="n"/>
+      <c r="AA197" s="10" t="n"/>
+      <c r="AB197" s="10" t="n"/>
+      <c r="AC197" s="10" t="n"/>
+      <c r="AD197" s="10" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="10" t="n"/>
@@ -4808,6 +5696,12 @@
       <c r="V198" s="10" t="n"/>
       <c r="W198" s="10" t="n"/>
       <c r="X198" s="10" t="n"/>
+      <c r="Y198" s="10" t="n"/>
+      <c r="Z198" s="10" t="n"/>
+      <c r="AA198" s="10" t="n"/>
+      <c r="AB198" s="10" t="n"/>
+      <c r="AC198" s="10" t="n"/>
+      <c r="AD198" s="10" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="10" t="n"/>
@@ -4834,6 +5728,12 @@
       <c r="V199" s="10" t="n"/>
       <c r="W199" s="10" t="n"/>
       <c r="X199" s="10" t="n"/>
+      <c r="Y199" s="10" t="n"/>
+      <c r="Z199" s="10" t="n"/>
+      <c r="AA199" s="10" t="n"/>
+      <c r="AB199" s="10" t="n"/>
+      <c r="AC199" s="10" t="n"/>
+      <c r="AD199" s="10" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="10" t="n"/>
@@ -4860,6 +5760,12 @@
       <c r="V200" s="10" t="n"/>
       <c r="W200" s="10" t="n"/>
       <c r="X200" s="10" t="n"/>
+      <c r="Y200" s="10" t="n"/>
+      <c r="Z200" s="10" t="n"/>
+      <c r="AA200" s="10" t="n"/>
+      <c r="AB200" s="10" t="n"/>
+      <c r="AC200" s="10" t="n"/>
+      <c r="AD200" s="10" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="10" t="n"/>
@@ -4886,6 +5792,12 @@
       <c r="V201" s="10" t="n"/>
       <c r="W201" s="10" t="n"/>
       <c r="X201" s="10" t="n"/>
+      <c r="Y201" s="10" t="n"/>
+      <c r="Z201" s="10" t="n"/>
+      <c r="AA201" s="10" t="n"/>
+      <c r="AB201" s="10" t="n"/>
+      <c r="AC201" s="10" t="n"/>
+      <c r="AD201" s="10" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="10" t="n"/>
@@ -4912,6 +5824,12 @@
       <c r="V202" s="10" t="n"/>
       <c r="W202" s="10" t="n"/>
       <c r="X202" s="10" t="n"/>
+      <c r="Y202" s="10" t="n"/>
+      <c r="Z202" s="10" t="n"/>
+      <c r="AA202" s="10" t="n"/>
+      <c r="AB202" s="10" t="n"/>
+      <c r="AC202" s="10" t="n"/>
+      <c r="AD202" s="10" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="10" t="n"/>
@@ -4938,6 +5856,12 @@
       <c r="V203" s="10" t="n"/>
       <c r="W203" s="10" t="n"/>
       <c r="X203" s="10" t="n"/>
+      <c r="Y203" s="10" t="n"/>
+      <c r="Z203" s="10" t="n"/>
+      <c r="AA203" s="10" t="n"/>
+      <c r="AB203" s="10" t="n"/>
+      <c r="AC203" s="10" t="n"/>
+      <c r="AD203" s="10" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="10" t="n"/>
@@ -4964,6 +5888,12 @@
       <c r="V204" s="10" t="n"/>
       <c r="W204" s="10" t="n"/>
       <c r="X204" s="10" t="n"/>
+      <c r="Y204" s="10" t="n"/>
+      <c r="Z204" s="10" t="n"/>
+      <c r="AA204" s="10" t="n"/>
+      <c r="AB204" s="10" t="n"/>
+      <c r="AC204" s="10" t="n"/>
+      <c r="AD204" s="10" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="10" t="n"/>
@@ -4990,6 +5920,12 @@
       <c r="V205" s="10" t="n"/>
       <c r="W205" s="10" t="n"/>
       <c r="X205" s="10" t="n"/>
+      <c r="Y205" s="10" t="n"/>
+      <c r="Z205" s="10" t="n"/>
+      <c r="AA205" s="10" t="n"/>
+      <c r="AB205" s="10" t="n"/>
+      <c r="AC205" s="10" t="n"/>
+      <c r="AD205" s="10" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="10" t="n"/>
@@ -5016,6 +5952,12 @@
       <c r="V206" s="10" t="n"/>
       <c r="W206" s="10" t="n"/>
       <c r="X206" s="10" t="n"/>
+      <c r="Y206" s="10" t="n"/>
+      <c r="Z206" s="10" t="n"/>
+      <c r="AA206" s="10" t="n"/>
+      <c r="AB206" s="10" t="n"/>
+      <c r="AC206" s="10" t="n"/>
+      <c r="AD206" s="10" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="10" t="n"/>
@@ -5042,6 +5984,12 @@
       <c r="V207" s="10" t="n"/>
       <c r="W207" s="10" t="n"/>
       <c r="X207" s="10" t="n"/>
+      <c r="Y207" s="10" t="n"/>
+      <c r="Z207" s="10" t="n"/>
+      <c r="AA207" s="10" t="n"/>
+      <c r="AB207" s="10" t="n"/>
+      <c r="AC207" s="10" t="n"/>
+      <c r="AD207" s="10" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="10" t="n"/>
@@ -5068,6 +6016,12 @@
       <c r="V208" s="10" t="n"/>
       <c r="W208" s="10" t="n"/>
       <c r="X208" s="10" t="n"/>
+      <c r="Y208" s="10" t="n"/>
+      <c r="Z208" s="10" t="n"/>
+      <c r="AA208" s="10" t="n"/>
+      <c r="AB208" s="10" t="n"/>
+      <c r="AC208" s="10" t="n"/>
+      <c r="AD208" s="10" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="10" t="n"/>
@@ -5094,6 +6048,12 @@
       <c r="V209" s="10" t="n"/>
       <c r="W209" s="10" t="n"/>
       <c r="X209" s="10" t="n"/>
+      <c r="Y209" s="10" t="n"/>
+      <c r="Z209" s="10" t="n"/>
+      <c r="AA209" s="10" t="n"/>
+      <c r="AB209" s="10" t="n"/>
+      <c r="AC209" s="10" t="n"/>
+      <c r="AD209" s="10" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="10" t="n"/>
@@ -5120,6 +6080,12 @@
       <c r="V210" s="10" t="n"/>
       <c r="W210" s="10" t="n"/>
       <c r="X210" s="10" t="n"/>
+      <c r="Y210" s="10" t="n"/>
+      <c r="Z210" s="10" t="n"/>
+      <c r="AA210" s="10" t="n"/>
+      <c r="AB210" s="10" t="n"/>
+      <c r="AC210" s="10" t="n"/>
+      <c r="AD210" s="10" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="10" t="n"/>
@@ -5146,6 +6112,12 @@
       <c r="V211" s="10" t="n"/>
       <c r="W211" s="10" t="n"/>
       <c r="X211" s="10" t="n"/>
+      <c r="Y211" s="10" t="n"/>
+      <c r="Z211" s="10" t="n"/>
+      <c r="AA211" s="10" t="n"/>
+      <c r="AB211" s="10" t="n"/>
+      <c r="AC211" s="10" t="n"/>
+      <c r="AD211" s="10" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="10" t="n"/>
@@ -5172,6 +6144,12 @@
       <c r="V212" s="10" t="n"/>
       <c r="W212" s="10" t="n"/>
       <c r="X212" s="10" t="n"/>
+      <c r="Y212" s="10" t="n"/>
+      <c r="Z212" s="10" t="n"/>
+      <c r="AA212" s="10" t="n"/>
+      <c r="AB212" s="10" t="n"/>
+      <c r="AC212" s="10" t="n"/>
+      <c r="AD212" s="10" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="10" t="n"/>
@@ -5198,6 +6176,12 @@
       <c r="V213" s="10" t="n"/>
       <c r="W213" s="10" t="n"/>
       <c r="X213" s="10" t="n"/>
+      <c r="Y213" s="10" t="n"/>
+      <c r="Z213" s="10" t="n"/>
+      <c r="AA213" s="10" t="n"/>
+      <c r="AB213" s="10" t="n"/>
+      <c r="AC213" s="10" t="n"/>
+      <c r="AD213" s="10" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="10" t="n"/>
@@ -5224,6 +6208,12 @@
       <c r="V214" s="10" t="n"/>
       <c r="W214" s="10" t="n"/>
       <c r="X214" s="10" t="n"/>
+      <c r="Y214" s="10" t="n"/>
+      <c r="Z214" s="10" t="n"/>
+      <c r="AA214" s="10" t="n"/>
+      <c r="AB214" s="10" t="n"/>
+      <c r="AC214" s="10" t="n"/>
+      <c r="AD214" s="10" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="10" t="n"/>
@@ -5250,6 +6240,12 @@
       <c r="V215" s="10" t="n"/>
       <c r="W215" s="10" t="n"/>
       <c r="X215" s="10" t="n"/>
+      <c r="Y215" s="10" t="n"/>
+      <c r="Z215" s="10" t="n"/>
+      <c r="AA215" s="10" t="n"/>
+      <c r="AB215" s="10" t="n"/>
+      <c r="AC215" s="10" t="n"/>
+      <c r="AD215" s="10" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="10" t="n"/>
@@ -5276,6 +6272,12 @@
       <c r="V216" s="10" t="n"/>
       <c r="W216" s="10" t="n"/>
       <c r="X216" s="10" t="n"/>
+      <c r="Y216" s="10" t="n"/>
+      <c r="Z216" s="10" t="n"/>
+      <c r="AA216" s="10" t="n"/>
+      <c r="AB216" s="10" t="n"/>
+      <c r="AC216" s="10" t="n"/>
+      <c r="AD216" s="10" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="10" t="n"/>
@@ -5302,6 +6304,12 @@
       <c r="V217" s="10" t="n"/>
       <c r="W217" s="10" t="n"/>
       <c r="X217" s="10" t="n"/>
+      <c r="Y217" s="10" t="n"/>
+      <c r="Z217" s="10" t="n"/>
+      <c r="AA217" s="10" t="n"/>
+      <c r="AB217" s="10" t="n"/>
+      <c r="AC217" s="10" t="n"/>
+      <c r="AD217" s="10" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="10" t="n"/>
@@ -5328,6 +6336,12 @@
       <c r="V218" s="10" t="n"/>
       <c r="W218" s="10" t="n"/>
       <c r="X218" s="10" t="n"/>
+      <c r="Y218" s="10" t="n"/>
+      <c r="Z218" s="10" t="n"/>
+      <c r="AA218" s="10" t="n"/>
+      <c r="AB218" s="10" t="n"/>
+      <c r="AC218" s="10" t="n"/>
+      <c r="AD218" s="10" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="10" t="n"/>
@@ -5354,6 +6368,12 @@
       <c r="V219" s="10" t="n"/>
       <c r="W219" s="10" t="n"/>
       <c r="X219" s="10" t="n"/>
+      <c r="Y219" s="10" t="n"/>
+      <c r="Z219" s="10" t="n"/>
+      <c r="AA219" s="10" t="n"/>
+      <c r="AB219" s="10" t="n"/>
+      <c r="AC219" s="10" t="n"/>
+      <c r="AD219" s="10" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="10" t="n"/>
@@ -5380,6 +6400,12 @@
       <c r="V220" s="10" t="n"/>
       <c r="W220" s="10" t="n"/>
       <c r="X220" s="10" t="n"/>
+      <c r="Y220" s="10" t="n"/>
+      <c r="Z220" s="10" t="n"/>
+      <c r="AA220" s="10" t="n"/>
+      <c r="AB220" s="10" t="n"/>
+      <c r="AC220" s="10" t="n"/>
+      <c r="AD220" s="10" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="10" t="n"/>
@@ -5406,6 +6432,12 @@
       <c r="V221" s="10" t="n"/>
       <c r="W221" s="10" t="n"/>
       <c r="X221" s="10" t="n"/>
+      <c r="Y221" s="10" t="n"/>
+      <c r="Z221" s="10" t="n"/>
+      <c r="AA221" s="10" t="n"/>
+      <c r="AB221" s="10" t="n"/>
+      <c r="AC221" s="10" t="n"/>
+      <c r="AD221" s="10" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="10" t="n"/>
@@ -5432,6 +6464,12 @@
       <c r="V222" s="10" t="n"/>
       <c r="W222" s="10" t="n"/>
       <c r="X222" s="10" t="n"/>
+      <c r="Y222" s="10" t="n"/>
+      <c r="Z222" s="10" t="n"/>
+      <c r="AA222" s="10" t="n"/>
+      <c r="AB222" s="10" t="n"/>
+      <c r="AC222" s="10" t="n"/>
+      <c r="AD222" s="10" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="10" t="n"/>
@@ -5458,6 +6496,12 @@
       <c r="V223" s="10" t="n"/>
       <c r="W223" s="10" t="n"/>
       <c r="X223" s="10" t="n"/>
+      <c r="Y223" s="10" t="n"/>
+      <c r="Z223" s="10" t="n"/>
+      <c r="AA223" s="10" t="n"/>
+      <c r="AB223" s="10" t="n"/>
+      <c r="AC223" s="10" t="n"/>
+      <c r="AD223" s="10" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="10" t="n"/>
@@ -5484,6 +6528,12 @@
       <c r="V224" s="10" t="n"/>
       <c r="W224" s="10" t="n"/>
       <c r="X224" s="10" t="n"/>
+      <c r="Y224" s="10" t="n"/>
+      <c r="Z224" s="10" t="n"/>
+      <c r="AA224" s="10" t="n"/>
+      <c r="AB224" s="10" t="n"/>
+      <c r="AC224" s="10" t="n"/>
+      <c r="AD224" s="10" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="10" t="n"/>
@@ -5510,6 +6560,12 @@
       <c r="V225" s="10" t="n"/>
       <c r="W225" s="10" t="n"/>
       <c r="X225" s="10" t="n"/>
+      <c r="Y225" s="10" t="n"/>
+      <c r="Z225" s="10" t="n"/>
+      <c r="AA225" s="10" t="n"/>
+      <c r="AB225" s="10" t="n"/>
+      <c r="AC225" s="10" t="n"/>
+      <c r="AD225" s="10" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="10" t="n"/>
@@ -5536,6 +6592,12 @@
       <c r="V226" s="10" t="n"/>
       <c r="W226" s="10" t="n"/>
       <c r="X226" s="10" t="n"/>
+      <c r="Y226" s="10" t="n"/>
+      <c r="Z226" s="10" t="n"/>
+      <c r="AA226" s="10" t="n"/>
+      <c r="AB226" s="10" t="n"/>
+      <c r="AC226" s="10" t="n"/>
+      <c r="AD226" s="10" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="10" t="n"/>
@@ -5562,6 +6624,12 @@
       <c r="V227" s="10" t="n"/>
       <c r="W227" s="10" t="n"/>
       <c r="X227" s="10" t="n"/>
+      <c r="Y227" s="10" t="n"/>
+      <c r="Z227" s="10" t="n"/>
+      <c r="AA227" s="10" t="n"/>
+      <c r="AB227" s="10" t="n"/>
+      <c r="AC227" s="10" t="n"/>
+      <c r="AD227" s="10" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="10" t="n"/>
@@ -5588,6 +6656,12 @@
       <c r="V228" s="10" t="n"/>
       <c r="W228" s="10" t="n"/>
       <c r="X228" s="10" t="n"/>
+      <c r="Y228" s="10" t="n"/>
+      <c r="Z228" s="10" t="n"/>
+      <c r="AA228" s="10" t="n"/>
+      <c r="AB228" s="10" t="n"/>
+      <c r="AC228" s="10" t="n"/>
+      <c r="AD228" s="10" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="10" t="n"/>
@@ -5614,6 +6688,12 @@
       <c r="V229" s="10" t="n"/>
       <c r="W229" s="10" t="n"/>
       <c r="X229" s="10" t="n"/>
+      <c r="Y229" s="10" t="n"/>
+      <c r="Z229" s="10" t="n"/>
+      <c r="AA229" s="10" t="n"/>
+      <c r="AB229" s="10" t="n"/>
+      <c r="AC229" s="10" t="n"/>
+      <c r="AD229" s="10" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="10" t="n"/>
@@ -5640,6 +6720,12 @@
       <c r="V230" s="10" t="n"/>
       <c r="W230" s="10" t="n"/>
       <c r="X230" s="10" t="n"/>
+      <c r="Y230" s="10" t="n"/>
+      <c r="Z230" s="10" t="n"/>
+      <c r="AA230" s="10" t="n"/>
+      <c r="AB230" s="10" t="n"/>
+      <c r="AC230" s="10" t="n"/>
+      <c r="AD230" s="10" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="10" t="n"/>
@@ -5666,6 +6752,12 @@
       <c r="V231" s="10" t="n"/>
       <c r="W231" s="10" t="n"/>
       <c r="X231" s="10" t="n"/>
+      <c r="Y231" s="10" t="n"/>
+      <c r="Z231" s="10" t="n"/>
+      <c r="AA231" s="10" t="n"/>
+      <c r="AB231" s="10" t="n"/>
+      <c r="AC231" s="10" t="n"/>
+      <c r="AD231" s="10" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="10" t="n"/>
@@ -5692,6 +6784,12 @@
       <c r="V232" s="10" t="n"/>
       <c r="W232" s="10" t="n"/>
       <c r="X232" s="10" t="n"/>
+      <c r="Y232" s="10" t="n"/>
+      <c r="Z232" s="10" t="n"/>
+      <c r="AA232" s="10" t="n"/>
+      <c r="AB232" s="10" t="n"/>
+      <c r="AC232" s="10" t="n"/>
+      <c r="AD232" s="10" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="10" t="n"/>
@@ -5718,6 +6816,12 @@
       <c r="V233" s="10" t="n"/>
       <c r="W233" s="10" t="n"/>
       <c r="X233" s="10" t="n"/>
+      <c r="Y233" s="10" t="n"/>
+      <c r="Z233" s="10" t="n"/>
+      <c r="AA233" s="10" t="n"/>
+      <c r="AB233" s="10" t="n"/>
+      <c r="AC233" s="10" t="n"/>
+      <c r="AD233" s="10" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="10" t="n"/>
@@ -5744,6 +6848,12 @@
       <c r="V234" s="10" t="n"/>
       <c r="W234" s="10" t="n"/>
       <c r="X234" s="10" t="n"/>
+      <c r="Y234" s="10" t="n"/>
+      <c r="Z234" s="10" t="n"/>
+      <c r="AA234" s="10" t="n"/>
+      <c r="AB234" s="10" t="n"/>
+      <c r="AC234" s="10" t="n"/>
+      <c r="AD234" s="10" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="10" t="n"/>
@@ -5770,6 +6880,12 @@
       <c r="V235" s="10" t="n"/>
       <c r="W235" s="10" t="n"/>
       <c r="X235" s="10" t="n"/>
+      <c r="Y235" s="10" t="n"/>
+      <c r="Z235" s="10" t="n"/>
+      <c r="AA235" s="10" t="n"/>
+      <c r="AB235" s="10" t="n"/>
+      <c r="AC235" s="10" t="n"/>
+      <c r="AD235" s="10" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="10" t="n"/>
@@ -5796,6 +6912,12 @@
       <c r="V236" s="10" t="n"/>
       <c r="W236" s="10" t="n"/>
       <c r="X236" s="10" t="n"/>
+      <c r="Y236" s="10" t="n"/>
+      <c r="Z236" s="10" t="n"/>
+      <c r="AA236" s="10" t="n"/>
+      <c r="AB236" s="10" t="n"/>
+      <c r="AC236" s="10" t="n"/>
+      <c r="AD236" s="10" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="10" t="n"/>
@@ -5822,6 +6944,12 @@
       <c r="V237" s="10" t="n"/>
       <c r="W237" s="10" t="n"/>
       <c r="X237" s="10" t="n"/>
+      <c r="Y237" s="10" t="n"/>
+      <c r="Z237" s="10" t="n"/>
+      <c r="AA237" s="10" t="n"/>
+      <c r="AB237" s="10" t="n"/>
+      <c r="AC237" s="10" t="n"/>
+      <c r="AD237" s="10" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="10" t="n"/>
@@ -5848,6 +6976,12 @@
       <c r="V238" s="10" t="n"/>
       <c r="W238" s="10" t="n"/>
       <c r="X238" s="10" t="n"/>
+      <c r="Y238" s="10" t="n"/>
+      <c r="Z238" s="10" t="n"/>
+      <c r="AA238" s="10" t="n"/>
+      <c r="AB238" s="10" t="n"/>
+      <c r="AC238" s="10" t="n"/>
+      <c r="AD238" s="10" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="10" t="n"/>
@@ -5874,6 +7008,12 @@
       <c r="V239" s="10" t="n"/>
       <c r="W239" s="10" t="n"/>
       <c r="X239" s="10" t="n"/>
+      <c r="Y239" s="10" t="n"/>
+      <c r="Z239" s="10" t="n"/>
+      <c r="AA239" s="10" t="n"/>
+      <c r="AB239" s="10" t="n"/>
+      <c r="AC239" s="10" t="n"/>
+      <c r="AD239" s="10" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="10" t="n"/>
@@ -5900,6 +7040,12 @@
       <c r="V240" s="10" t="n"/>
       <c r="W240" s="10" t="n"/>
       <c r="X240" s="10" t="n"/>
+      <c r="Y240" s="10" t="n"/>
+      <c r="Z240" s="10" t="n"/>
+      <c r="AA240" s="10" t="n"/>
+      <c r="AB240" s="10" t="n"/>
+      <c r="AC240" s="10" t="n"/>
+      <c r="AD240" s="10" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="10" t="n"/>
@@ -5926,6 +7072,12 @@
       <c r="V241" s="10" t="n"/>
       <c r="W241" s="10" t="n"/>
       <c r="X241" s="10" t="n"/>
+      <c r="Y241" s="10" t="n"/>
+      <c r="Z241" s="10" t="n"/>
+      <c r="AA241" s="10" t="n"/>
+      <c r="AB241" s="10" t="n"/>
+      <c r="AC241" s="10" t="n"/>
+      <c r="AD241" s="10" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="10" t="n"/>
@@ -5952,6 +7104,12 @@
       <c r="V242" s="10" t="n"/>
       <c r="W242" s="10" t="n"/>
       <c r="X242" s="10" t="n"/>
+      <c r="Y242" s="10" t="n"/>
+      <c r="Z242" s="10" t="n"/>
+      <c r="AA242" s="10" t="n"/>
+      <c r="AB242" s="10" t="n"/>
+      <c r="AC242" s="10" t="n"/>
+      <c r="AD242" s="10" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="10" t="n"/>
@@ -5978,6 +7136,12 @@
       <c r="V243" s="10" t="n"/>
       <c r="W243" s="10" t="n"/>
       <c r="X243" s="10" t="n"/>
+      <c r="Y243" s="10" t="n"/>
+      <c r="Z243" s="10" t="n"/>
+      <c r="AA243" s="10" t="n"/>
+      <c r="AB243" s="10" t="n"/>
+      <c r="AC243" s="10" t="n"/>
+      <c r="AD243" s="10" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="10" t="n"/>
@@ -6004,6 +7168,12 @@
       <c r="V244" s="10" t="n"/>
       <c r="W244" s="10" t="n"/>
       <c r="X244" s="10" t="n"/>
+      <c r="Y244" s="10" t="n"/>
+      <c r="Z244" s="10" t="n"/>
+      <c r="AA244" s="10" t="n"/>
+      <c r="AB244" s="10" t="n"/>
+      <c r="AC244" s="10" t="n"/>
+      <c r="AD244" s="10" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="10" t="n"/>
@@ -6030,6 +7200,12 @@
       <c r="V245" s="10" t="n"/>
       <c r="W245" s="10" t="n"/>
       <c r="X245" s="10" t="n"/>
+      <c r="Y245" s="10" t="n"/>
+      <c r="Z245" s="10" t="n"/>
+      <c r="AA245" s="10" t="n"/>
+      <c r="AB245" s="10" t="n"/>
+      <c r="AC245" s="10" t="n"/>
+      <c r="AD245" s="10" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="10" t="n"/>
@@ -6056,6 +7232,12 @@
       <c r="V246" s="10" t="n"/>
       <c r="W246" s="10" t="n"/>
       <c r="X246" s="10" t="n"/>
+      <c r="Y246" s="10" t="n"/>
+      <c r="Z246" s="10" t="n"/>
+      <c r="AA246" s="10" t="n"/>
+      <c r="AB246" s="10" t="n"/>
+      <c r="AC246" s="10" t="n"/>
+      <c r="AD246" s="10" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="10" t="n"/>
@@ -6082,6 +7264,12 @@
       <c r="V247" s="10" t="n"/>
       <c r="W247" s="10" t="n"/>
       <c r="X247" s="10" t="n"/>
+      <c r="Y247" s="10" t="n"/>
+      <c r="Z247" s="10" t="n"/>
+      <c r="AA247" s="10" t="n"/>
+      <c r="AB247" s="10" t="n"/>
+      <c r="AC247" s="10" t="n"/>
+      <c r="AD247" s="10" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="10" t="n"/>
@@ -6108,6 +7296,12 @@
       <c r="V248" s="10" t="n"/>
       <c r="W248" s="10" t="n"/>
       <c r="X248" s="10" t="n"/>
+      <c r="Y248" s="10" t="n"/>
+      <c r="Z248" s="10" t="n"/>
+      <c r="AA248" s="10" t="n"/>
+      <c r="AB248" s="10" t="n"/>
+      <c r="AC248" s="10" t="n"/>
+      <c r="AD248" s="10" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="10" t="n"/>
@@ -6134,6 +7328,12 @@
       <c r="V249" s="10" t="n"/>
       <c r="W249" s="10" t="n"/>
       <c r="X249" s="10" t="n"/>
+      <c r="Y249" s="10" t="n"/>
+      <c r="Z249" s="10" t="n"/>
+      <c r="AA249" s="10" t="n"/>
+      <c r="AB249" s="10" t="n"/>
+      <c r="AC249" s="10" t="n"/>
+      <c r="AD249" s="10" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="10" t="n"/>
@@ -6160,6 +7360,12 @@
       <c r="V250" s="10" t="n"/>
       <c r="W250" s="10" t="n"/>
       <c r="X250" s="10" t="n"/>
+      <c r="Y250" s="10" t="n"/>
+      <c r="Z250" s="10" t="n"/>
+      <c r="AA250" s="10" t="n"/>
+      <c r="AB250" s="10" t="n"/>
+      <c r="AC250" s="10" t="n"/>
+      <c r="AD250" s="10" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="10" t="n"/>
@@ -6186,6 +7392,12 @@
       <c r="V251" s="10" t="n"/>
       <c r="W251" s="10" t="n"/>
       <c r="X251" s="10" t="n"/>
+      <c r="Y251" s="10" t="n"/>
+      <c r="Z251" s="10" t="n"/>
+      <c r="AA251" s="10" t="n"/>
+      <c r="AB251" s="10" t="n"/>
+      <c r="AC251" s="10" t="n"/>
+      <c r="AD251" s="10" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="10" t="n"/>
@@ -6212,6 +7424,12 @@
       <c r="V252" s="10" t="n"/>
       <c r="W252" s="10" t="n"/>
       <c r="X252" s="10" t="n"/>
+      <c r="Y252" s="10" t="n"/>
+      <c r="Z252" s="10" t="n"/>
+      <c r="AA252" s="10" t="n"/>
+      <c r="AB252" s="10" t="n"/>
+      <c r="AC252" s="10" t="n"/>
+      <c r="AD252" s="10" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="10" t="n"/>
@@ -6238,6 +7456,12 @@
       <c r="V253" s="10" t="n"/>
       <c r="W253" s="10" t="n"/>
       <c r="X253" s="10" t="n"/>
+      <c r="Y253" s="10" t="n"/>
+      <c r="Z253" s="10" t="n"/>
+      <c r="AA253" s="10" t="n"/>
+      <c r="AB253" s="10" t="n"/>
+      <c r="AC253" s="10" t="n"/>
+      <c r="AD253" s="10" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="10" t="n"/>
@@ -6264,6 +7488,12 @@
       <c r="V254" s="10" t="n"/>
       <c r="W254" s="10" t="n"/>
       <c r="X254" s="10" t="n"/>
+      <c r="Y254" s="10" t="n"/>
+      <c r="Z254" s="10" t="n"/>
+      <c r="AA254" s="10" t="n"/>
+      <c r="AB254" s="10" t="n"/>
+      <c r="AC254" s="10" t="n"/>
+      <c r="AD254" s="10" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="10" t="n"/>
@@ -6290,6 +7520,12 @@
       <c r="V255" s="10" t="n"/>
       <c r="W255" s="10" t="n"/>
       <c r="X255" s="10" t="n"/>
+      <c r="Y255" s="10" t="n"/>
+      <c r="Z255" s="10" t="n"/>
+      <c r="AA255" s="10" t="n"/>
+      <c r="AB255" s="10" t="n"/>
+      <c r="AC255" s="10" t="n"/>
+      <c r="AD255" s="10" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="10" t="n"/>
@@ -6316,6 +7552,12 @@
       <c r="V256" s="10" t="n"/>
       <c r="W256" s="10" t="n"/>
       <c r="X256" s="10" t="n"/>
+      <c r="Y256" s="10" t="n"/>
+      <c r="Z256" s="10" t="n"/>
+      <c r="AA256" s="10" t="n"/>
+      <c r="AB256" s="10" t="n"/>
+      <c r="AC256" s="10" t="n"/>
+      <c r="AD256" s="10" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="10" t="n"/>
@@ -6342,6 +7584,12 @@
       <c r="V257" s="10" t="n"/>
       <c r="W257" s="10" t="n"/>
       <c r="X257" s="10" t="n"/>
+      <c r="Y257" s="10" t="n"/>
+      <c r="Z257" s="10" t="n"/>
+      <c r="AA257" s="10" t="n"/>
+      <c r="AB257" s="10" t="n"/>
+      <c r="AC257" s="10" t="n"/>
+      <c r="AD257" s="10" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="10" t="n"/>
@@ -6368,6 +7616,12 @@
       <c r="V258" s="10" t="n"/>
       <c r="W258" s="10" t="n"/>
       <c r="X258" s="10" t="n"/>
+      <c r="Y258" s="10" t="n"/>
+      <c r="Z258" s="10" t="n"/>
+      <c r="AA258" s="10" t="n"/>
+      <c r="AB258" s="10" t="n"/>
+      <c r="AC258" s="10" t="n"/>
+      <c r="AD258" s="10" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="10" t="n"/>
@@ -6394,6 +7648,12 @@
       <c r="V259" s="10" t="n"/>
       <c r="W259" s="10" t="n"/>
       <c r="X259" s="10" t="n"/>
+      <c r="Y259" s="10" t="n"/>
+      <c r="Z259" s="10" t="n"/>
+      <c r="AA259" s="10" t="n"/>
+      <c r="AB259" s="10" t="n"/>
+      <c r="AC259" s="10" t="n"/>
+      <c r="AD259" s="10" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="10" t="n"/>
@@ -6420,6 +7680,12 @@
       <c r="V260" s="10" t="n"/>
       <c r="W260" s="10" t="n"/>
       <c r="X260" s="10" t="n"/>
+      <c r="Y260" s="10" t="n"/>
+      <c r="Z260" s="10" t="n"/>
+      <c r="AA260" s="10" t="n"/>
+      <c r="AB260" s="10" t="n"/>
+      <c r="AC260" s="10" t="n"/>
+      <c r="AD260" s="10" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="10" t="n"/>
@@ -6446,6 +7712,12 @@
       <c r="V261" s="10" t="n"/>
       <c r="W261" s="10" t="n"/>
       <c r="X261" s="10" t="n"/>
+      <c r="Y261" s="10" t="n"/>
+      <c r="Z261" s="10" t="n"/>
+      <c r="AA261" s="10" t="n"/>
+      <c r="AB261" s="10" t="n"/>
+      <c r="AC261" s="10" t="n"/>
+      <c r="AD261" s="10" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="10" t="n"/>
@@ -6472,6 +7744,12 @@
       <c r="V262" s="10" t="n"/>
       <c r="W262" s="10" t="n"/>
       <c r="X262" s="10" t="n"/>
+      <c r="Y262" s="10" t="n"/>
+      <c r="Z262" s="10" t="n"/>
+      <c r="AA262" s="10" t="n"/>
+      <c r="AB262" s="10" t="n"/>
+      <c r="AC262" s="10" t="n"/>
+      <c r="AD262" s="10" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="10" t="n"/>
@@ -6498,6 +7776,12 @@
       <c r="V263" s="10" t="n"/>
       <c r="W263" s="10" t="n"/>
       <c r="X263" s="10" t="n"/>
+      <c r="Y263" s="10" t="n"/>
+      <c r="Z263" s="10" t="n"/>
+      <c r="AA263" s="10" t="n"/>
+      <c r="AB263" s="10" t="n"/>
+      <c r="AC263" s="10" t="n"/>
+      <c r="AD263" s="10" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="10" t="n"/>
@@ -6524,6 +7808,12 @@
       <c r="V264" s="10" t="n"/>
       <c r="W264" s="10" t="n"/>
       <c r="X264" s="10" t="n"/>
+      <c r="Y264" s="10" t="n"/>
+      <c r="Z264" s="10" t="n"/>
+      <c r="AA264" s="10" t="n"/>
+      <c r="AB264" s="10" t="n"/>
+      <c r="AC264" s="10" t="n"/>
+      <c r="AD264" s="10" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="10" t="n"/>
@@ -6550,6 +7840,12 @@
       <c r="V265" s="10" t="n"/>
       <c r="W265" s="10" t="n"/>
       <c r="X265" s="10" t="n"/>
+      <c r="Y265" s="10" t="n"/>
+      <c r="Z265" s="10" t="n"/>
+      <c r="AA265" s="10" t="n"/>
+      <c r="AB265" s="10" t="n"/>
+      <c r="AC265" s="10" t="n"/>
+      <c r="AD265" s="10" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="10" t="n"/>
@@ -6576,6 +7872,12 @@
       <c r="V266" s="10" t="n"/>
       <c r="W266" s="10" t="n"/>
       <c r="X266" s="10" t="n"/>
+      <c r="Y266" s="10" t="n"/>
+      <c r="Z266" s="10" t="n"/>
+      <c r="AA266" s="10" t="n"/>
+      <c r="AB266" s="10" t="n"/>
+      <c r="AC266" s="10" t="n"/>
+      <c r="AD266" s="10" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="10" t="n"/>
@@ -6602,6 +7904,12 @@
       <c r="V267" s="10" t="n"/>
       <c r="W267" s="10" t="n"/>
       <c r="X267" s="10" t="n"/>
+      <c r="Y267" s="10" t="n"/>
+      <c r="Z267" s="10" t="n"/>
+      <c r="AA267" s="10" t="n"/>
+      <c r="AB267" s="10" t="n"/>
+      <c r="AC267" s="10" t="n"/>
+      <c r="AD267" s="10" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="10" t="n"/>
@@ -6628,6 +7936,12 @@
       <c r="V268" s="10" t="n"/>
       <c r="W268" s="10" t="n"/>
       <c r="X268" s="10" t="n"/>
+      <c r="Y268" s="10" t="n"/>
+      <c r="Z268" s="10" t="n"/>
+      <c r="AA268" s="10" t="n"/>
+      <c r="AB268" s="10" t="n"/>
+      <c r="AC268" s="10" t="n"/>
+      <c r="AD268" s="10" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="10" t="n"/>
@@ -6654,6 +7968,12 @@
       <c r="V269" s="10" t="n"/>
       <c r="W269" s="10" t="n"/>
       <c r="X269" s="10" t="n"/>
+      <c r="Y269" s="10" t="n"/>
+      <c r="Z269" s="10" t="n"/>
+      <c r="AA269" s="10" t="n"/>
+      <c r="AB269" s="10" t="n"/>
+      <c r="AC269" s="10" t="n"/>
+      <c r="AD269" s="10" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="10" t="n"/>
@@ -6680,6 +8000,12 @@
       <c r="V270" s="10" t="n"/>
       <c r="W270" s="10" t="n"/>
       <c r="X270" s="10" t="n"/>
+      <c r="Y270" s="10" t="n"/>
+      <c r="Z270" s="10" t="n"/>
+      <c r="AA270" s="10" t="n"/>
+      <c r="AB270" s="10" t="n"/>
+      <c r="AC270" s="10" t="n"/>
+      <c r="AD270" s="10" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="10" t="n"/>
@@ -6706,6 +8032,12 @@
       <c r="V271" s="10" t="n"/>
       <c r="W271" s="10" t="n"/>
       <c r="X271" s="10" t="n"/>
+      <c r="Y271" s="10" t="n"/>
+      <c r="Z271" s="10" t="n"/>
+      <c r="AA271" s="10" t="n"/>
+      <c r="AB271" s="10" t="n"/>
+      <c r="AC271" s="10" t="n"/>
+      <c r="AD271" s="10" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="10" t="n"/>
@@ -6732,6 +8064,12 @@
       <c r="V272" s="10" t="n"/>
       <c r="W272" s="10" t="n"/>
       <c r="X272" s="10" t="n"/>
+      <c r="Y272" s="10" t="n"/>
+      <c r="Z272" s="10" t="n"/>
+      <c r="AA272" s="10" t="n"/>
+      <c r="AB272" s="10" t="n"/>
+      <c r="AC272" s="10" t="n"/>
+      <c r="AD272" s="10" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="10" t="n"/>
@@ -6758,6 +8096,12 @@
       <c r="V273" s="10" t="n"/>
       <c r="W273" s="10" t="n"/>
       <c r="X273" s="10" t="n"/>
+      <c r="Y273" s="10" t="n"/>
+      <c r="Z273" s="10" t="n"/>
+      <c r="AA273" s="10" t="n"/>
+      <c r="AB273" s="10" t="n"/>
+      <c r="AC273" s="10" t="n"/>
+      <c r="AD273" s="10" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="10" t="n"/>
@@ -6784,6 +8128,12 @@
       <c r="V274" s="10" t="n"/>
       <c r="W274" s="10" t="n"/>
       <c r="X274" s="10" t="n"/>
+      <c r="Y274" s="10" t="n"/>
+      <c r="Z274" s="10" t="n"/>
+      <c r="AA274" s="10" t="n"/>
+      <c r="AB274" s="10" t="n"/>
+      <c r="AC274" s="10" t="n"/>
+      <c r="AD274" s="10" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="10" t="n"/>
@@ -6810,6 +8160,12 @@
       <c r="V275" s="10" t="n"/>
       <c r="W275" s="10" t="n"/>
       <c r="X275" s="10" t="n"/>
+      <c r="Y275" s="10" t="n"/>
+      <c r="Z275" s="10" t="n"/>
+      <c r="AA275" s="10" t="n"/>
+      <c r="AB275" s="10" t="n"/>
+      <c r="AC275" s="10" t="n"/>
+      <c r="AD275" s="10" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="10" t="n"/>
@@ -6836,6 +8192,12 @@
       <c r="V276" s="10" t="n"/>
       <c r="W276" s="10" t="n"/>
       <c r="X276" s="10" t="n"/>
+      <c r="Y276" s="10" t="n"/>
+      <c r="Z276" s="10" t="n"/>
+      <c r="AA276" s="10" t="n"/>
+      <c r="AB276" s="10" t="n"/>
+      <c r="AC276" s="10" t="n"/>
+      <c r="AD276" s="10" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="10" t="n"/>
@@ -6862,6 +8224,12 @@
       <c r="V277" s="10" t="n"/>
       <c r="W277" s="10" t="n"/>
       <c r="X277" s="10" t="n"/>
+      <c r="Y277" s="10" t="n"/>
+      <c r="Z277" s="10" t="n"/>
+      <c r="AA277" s="10" t="n"/>
+      <c r="AB277" s="10" t="n"/>
+      <c r="AC277" s="10" t="n"/>
+      <c r="AD277" s="10" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="10" t="n"/>
@@ -6888,6 +8256,12 @@
       <c r="V278" s="10" t="n"/>
       <c r="W278" s="10" t="n"/>
       <c r="X278" s="10" t="n"/>
+      <c r="Y278" s="10" t="n"/>
+      <c r="Z278" s="10" t="n"/>
+      <c r="AA278" s="10" t="n"/>
+      <c r="AB278" s="10" t="n"/>
+      <c r="AC278" s="10" t="n"/>
+      <c r="AD278" s="10" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="10" t="n"/>
@@ -6914,6 +8288,12 @@
       <c r="V279" s="10" t="n"/>
       <c r="W279" s="10" t="n"/>
       <c r="X279" s="10" t="n"/>
+      <c r="Y279" s="10" t="n"/>
+      <c r="Z279" s="10" t="n"/>
+      <c r="AA279" s="10" t="n"/>
+      <c r="AB279" s="10" t="n"/>
+      <c r="AC279" s="10" t="n"/>
+      <c r="AD279" s="10" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="10" t="n"/>
@@ -6940,6 +8320,12 @@
       <c r="V280" s="10" t="n"/>
       <c r="W280" s="10" t="n"/>
       <c r="X280" s="10" t="n"/>
+      <c r="Y280" s="10" t="n"/>
+      <c r="Z280" s="10" t="n"/>
+      <c r="AA280" s="10" t="n"/>
+      <c r="AB280" s="10" t="n"/>
+      <c r="AC280" s="10" t="n"/>
+      <c r="AD280" s="10" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="10" t="n"/>
@@ -6966,6 +8352,12 @@
       <c r="V281" s="10" t="n"/>
       <c r="W281" s="10" t="n"/>
       <c r="X281" s="10" t="n"/>
+      <c r="Y281" s="10" t="n"/>
+      <c r="Z281" s="10" t="n"/>
+      <c r="AA281" s="10" t="n"/>
+      <c r="AB281" s="10" t="n"/>
+      <c r="AC281" s="10" t="n"/>
+      <c r="AD281" s="10" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="10" t="n"/>
@@ -6992,6 +8384,12 @@
       <c r="V282" s="10" t="n"/>
       <c r="W282" s="10" t="n"/>
       <c r="X282" s="10" t="n"/>
+      <c r="Y282" s="10" t="n"/>
+      <c r="Z282" s="10" t="n"/>
+      <c r="AA282" s="10" t="n"/>
+      <c r="AB282" s="10" t="n"/>
+      <c r="AC282" s="10" t="n"/>
+      <c r="AD282" s="10" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="10" t="n"/>
@@ -7018,6 +8416,12 @@
       <c r="V283" s="10" t="n"/>
       <c r="W283" s="10" t="n"/>
       <c r="X283" s="10" t="n"/>
+      <c r="Y283" s="10" t="n"/>
+      <c r="Z283" s="10" t="n"/>
+      <c r="AA283" s="10" t="n"/>
+      <c r="AB283" s="10" t="n"/>
+      <c r="AC283" s="10" t="n"/>
+      <c r="AD283" s="10" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="10" t="n"/>
@@ -7044,6 +8448,12 @@
       <c r="V284" s="10" t="n"/>
       <c r="W284" s="10" t="n"/>
       <c r="X284" s="10" t="n"/>
+      <c r="Y284" s="10" t="n"/>
+      <c r="Z284" s="10" t="n"/>
+      <c r="AA284" s="10" t="n"/>
+      <c r="AB284" s="10" t="n"/>
+      <c r="AC284" s="10" t="n"/>
+      <c r="AD284" s="10" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="10" t="n"/>
@@ -7070,6 +8480,12 @@
       <c r="V285" s="10" t="n"/>
       <c r="W285" s="10" t="n"/>
       <c r="X285" s="10" t="n"/>
+      <c r="Y285" s="10" t="n"/>
+      <c r="Z285" s="10" t="n"/>
+      <c r="AA285" s="10" t="n"/>
+      <c r="AB285" s="10" t="n"/>
+      <c r="AC285" s="10" t="n"/>
+      <c r="AD285" s="10" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="10" t="n"/>
@@ -7096,6 +8512,12 @@
       <c r="V286" s="10" t="n"/>
       <c r="W286" s="10" t="n"/>
       <c r="X286" s="10" t="n"/>
+      <c r="Y286" s="10" t="n"/>
+      <c r="Z286" s="10" t="n"/>
+      <c r="AA286" s="10" t="n"/>
+      <c r="AB286" s="10" t="n"/>
+      <c r="AC286" s="10" t="n"/>
+      <c r="AD286" s="10" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="10" t="n"/>
@@ -7122,6 +8544,12 @@
       <c r="V287" s="10" t="n"/>
       <c r="W287" s="10" t="n"/>
       <c r="X287" s="10" t="n"/>
+      <c r="Y287" s="10" t="n"/>
+      <c r="Z287" s="10" t="n"/>
+      <c r="AA287" s="10" t="n"/>
+      <c r="AB287" s="10" t="n"/>
+      <c r="AC287" s="10" t="n"/>
+      <c r="AD287" s="10" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="10" t="n"/>
@@ -7148,6 +8576,12 @@
       <c r="V288" s="10" t="n"/>
       <c r="W288" s="10" t="n"/>
       <c r="X288" s="10" t="n"/>
+      <c r="Y288" s="10" t="n"/>
+      <c r="Z288" s="10" t="n"/>
+      <c r="AA288" s="10" t="n"/>
+      <c r="AB288" s="10" t="n"/>
+      <c r="AC288" s="10" t="n"/>
+      <c r="AD288" s="10" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="10" t="n"/>
@@ -7174,6 +8608,12 @@
       <c r="V289" s="10" t="n"/>
       <c r="W289" s="10" t="n"/>
       <c r="X289" s="10" t="n"/>
+      <c r="Y289" s="10" t="n"/>
+      <c r="Z289" s="10" t="n"/>
+      <c r="AA289" s="10" t="n"/>
+      <c r="AB289" s="10" t="n"/>
+      <c r="AC289" s="10" t="n"/>
+      <c r="AD289" s="10" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="10" t="n"/>
@@ -7200,6 +8640,12 @@
       <c r="V290" s="10" t="n"/>
       <c r="W290" s="10" t="n"/>
       <c r="X290" s="10" t="n"/>
+      <c r="Y290" s="10" t="n"/>
+      <c r="Z290" s="10" t="n"/>
+      <c r="AA290" s="10" t="n"/>
+      <c r="AB290" s="10" t="n"/>
+      <c r="AC290" s="10" t="n"/>
+      <c r="AD290" s="10" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="10" t="n"/>
@@ -7226,6 +8672,12 @@
       <c r="V291" s="10" t="n"/>
       <c r="W291" s="10" t="n"/>
       <c r="X291" s="10" t="n"/>
+      <c r="Y291" s="10" t="n"/>
+      <c r="Z291" s="10" t="n"/>
+      <c r="AA291" s="10" t="n"/>
+      <c r="AB291" s="10" t="n"/>
+      <c r="AC291" s="10" t="n"/>
+      <c r="AD291" s="10" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="10" t="n"/>
@@ -7252,6 +8704,12 @@
       <c r="V292" s="10" t="n"/>
       <c r="W292" s="10" t="n"/>
       <c r="X292" s="10" t="n"/>
+      <c r="Y292" s="10" t="n"/>
+      <c r="Z292" s="10" t="n"/>
+      <c r="AA292" s="10" t="n"/>
+      <c r="AB292" s="10" t="n"/>
+      <c r="AC292" s="10" t="n"/>
+      <c r="AD292" s="10" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="10" t="n"/>
@@ -7278,6 +8736,12 @@
       <c r="V293" s="10" t="n"/>
       <c r="W293" s="10" t="n"/>
       <c r="X293" s="10" t="n"/>
+      <c r="Y293" s="10" t="n"/>
+      <c r="Z293" s="10" t="n"/>
+      <c r="AA293" s="10" t="n"/>
+      <c r="AB293" s="10" t="n"/>
+      <c r="AC293" s="10" t="n"/>
+      <c r="AD293" s="10" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="10" t="n"/>
@@ -7304,6 +8768,12 @@
       <c r="V294" s="10" t="n"/>
       <c r="W294" s="10" t="n"/>
       <c r="X294" s="10" t="n"/>
+      <c r="Y294" s="10" t="n"/>
+      <c r="Z294" s="10" t="n"/>
+      <c r="AA294" s="10" t="n"/>
+      <c r="AB294" s="10" t="n"/>
+      <c r="AC294" s="10" t="n"/>
+      <c r="AD294" s="10" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="10" t="n"/>
@@ -7330,6 +8800,12 @@
       <c r="V295" s="10" t="n"/>
       <c r="W295" s="10" t="n"/>
       <c r="X295" s="10" t="n"/>
+      <c r="Y295" s="10" t="n"/>
+      <c r="Z295" s="10" t="n"/>
+      <c r="AA295" s="10" t="n"/>
+      <c r="AB295" s="10" t="n"/>
+      <c r="AC295" s="10" t="n"/>
+      <c r="AD295" s="10" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="10" t="n"/>
@@ -7356,6 +8832,12 @@
       <c r="V296" s="10" t="n"/>
       <c r="W296" s="10" t="n"/>
       <c r="X296" s="10" t="n"/>
+      <c r="Y296" s="10" t="n"/>
+      <c r="Z296" s="10" t="n"/>
+      <c r="AA296" s="10" t="n"/>
+      <c r="AB296" s="10" t="n"/>
+      <c r="AC296" s="10" t="n"/>
+      <c r="AD296" s="10" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="10" t="n"/>
@@ -7382,6 +8864,12 @@
       <c r="V297" s="10" t="n"/>
       <c r="W297" s="10" t="n"/>
       <c r="X297" s="10" t="n"/>
+      <c r="Y297" s="10" t="n"/>
+      <c r="Z297" s="10" t="n"/>
+      <c r="AA297" s="10" t="n"/>
+      <c r="AB297" s="10" t="n"/>
+      <c r="AC297" s="10" t="n"/>
+      <c r="AD297" s="10" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="10" t="n"/>
@@ -7408,6 +8896,12 @@
       <c r="V298" s="10" t="n"/>
       <c r="W298" s="10" t="n"/>
       <c r="X298" s="10" t="n"/>
+      <c r="Y298" s="10" t="n"/>
+      <c r="Z298" s="10" t="n"/>
+      <c r="AA298" s="10" t="n"/>
+      <c r="AB298" s="10" t="n"/>
+      <c r="AC298" s="10" t="n"/>
+      <c r="AD298" s="10" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="10" t="n"/>
@@ -7434,6 +8928,12 @@
       <c r="V299" s="10" t="n"/>
       <c r="W299" s="10" t="n"/>
       <c r="X299" s="10" t="n"/>
+      <c r="Y299" s="10" t="n"/>
+      <c r="Z299" s="10" t="n"/>
+      <c r="AA299" s="10" t="n"/>
+      <c r="AB299" s="10" t="n"/>
+      <c r="AC299" s="10" t="n"/>
+      <c r="AD299" s="10" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="10" t="n"/>
@@ -7460,6 +8960,12 @@
       <c r="V300" s="10" t="n"/>
       <c r="W300" s="10" t="n"/>
       <c r="X300" s="10" t="n"/>
+      <c r="Y300" s="10" t="n"/>
+      <c r="Z300" s="10" t="n"/>
+      <c r="AA300" s="10" t="n"/>
+      <c r="AB300" s="10" t="n"/>
+      <c r="AC300" s="10" t="n"/>
+      <c r="AD300" s="10" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="10" t="n"/>
@@ -7486,6 +8992,12 @@
       <c r="V301" s="10" t="n"/>
       <c r="W301" s="10" t="n"/>
       <c r="X301" s="10" t="n"/>
+      <c r="Y301" s="10" t="n"/>
+      <c r="Z301" s="10" t="n"/>
+      <c r="AA301" s="10" t="n"/>
+      <c r="AB301" s="10" t="n"/>
+      <c r="AC301" s="10" t="n"/>
+      <c r="AD301" s="10" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="10" t="n"/>
@@ -7512,6 +9024,12 @@
       <c r="V302" s="10" t="n"/>
       <c r="W302" s="10" t="n"/>
       <c r="X302" s="10" t="n"/>
+      <c r="Y302" s="10" t="n"/>
+      <c r="Z302" s="10" t="n"/>
+      <c r="AA302" s="10" t="n"/>
+      <c r="AB302" s="10" t="n"/>
+      <c r="AC302" s="10" t="n"/>
+      <c r="AD302" s="10" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="10" t="n"/>
@@ -7538,6 +9056,12 @@
       <c r="V303" s="10" t="n"/>
       <c r="W303" s="10" t="n"/>
       <c r="X303" s="10" t="n"/>
+      <c r="Y303" s="10" t="n"/>
+      <c r="Z303" s="10" t="n"/>
+      <c r="AA303" s="10" t="n"/>
+      <c r="AB303" s="10" t="n"/>
+      <c r="AC303" s="10" t="n"/>
+      <c r="AD303" s="10" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="10" t="n"/>
@@ -7564,6 +9088,12 @@
       <c r="V304" s="10" t="n"/>
       <c r="W304" s="10" t="n"/>
       <c r="X304" s="10" t="n"/>
+      <c r="Y304" s="10" t="n"/>
+      <c r="Z304" s="10" t="n"/>
+      <c r="AA304" s="10" t="n"/>
+      <c r="AB304" s="10" t="n"/>
+      <c r="AC304" s="10" t="n"/>
+      <c r="AD304" s="10" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="10" t="n"/>
@@ -7590,6 +9120,12 @@
       <c r="V305" s="10" t="n"/>
       <c r="W305" s="10" t="n"/>
       <c r="X305" s="10" t="n"/>
+      <c r="Y305" s="10" t="n"/>
+      <c r="Z305" s="10" t="n"/>
+      <c r="AA305" s="10" t="n"/>
+      <c r="AB305" s="10" t="n"/>
+      <c r="AC305" s="10" t="n"/>
+      <c r="AD305" s="10" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="10" t="n"/>
@@ -7616,6 +9152,12 @@
       <c r="V306" s="10" t="n"/>
       <c r="W306" s="10" t="n"/>
       <c r="X306" s="10" t="n"/>
+      <c r="Y306" s="10" t="n"/>
+      <c r="Z306" s="10" t="n"/>
+      <c r="AA306" s="10" t="n"/>
+      <c r="AB306" s="10" t="n"/>
+      <c r="AC306" s="10" t="n"/>
+      <c r="AD306" s="10" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="10" t="n"/>
@@ -7642,6 +9184,12 @@
       <c r="V307" s="10" t="n"/>
       <c r="W307" s="10" t="n"/>
       <c r="X307" s="10" t="n"/>
+      <c r="Y307" s="10" t="n"/>
+      <c r="Z307" s="10" t="n"/>
+      <c r="AA307" s="10" t="n"/>
+      <c r="AB307" s="10" t="n"/>
+      <c r="AC307" s="10" t="n"/>
+      <c r="AD307" s="10" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="10" t="n"/>
@@ -7668,6 +9216,12 @@
       <c r="V308" s="10" t="n"/>
       <c r="W308" s="10" t="n"/>
       <c r="X308" s="10" t="n"/>
+      <c r="Y308" s="10" t="n"/>
+      <c r="Z308" s="10" t="n"/>
+      <c r="AA308" s="10" t="n"/>
+      <c r="AB308" s="10" t="n"/>
+      <c r="AC308" s="10" t="n"/>
+      <c r="AD308" s="10" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="10" t="n"/>
@@ -7694,6 +9248,12 @@
       <c r="V309" s="10" t="n"/>
       <c r="W309" s="10" t="n"/>
       <c r="X309" s="10" t="n"/>
+      <c r="Y309" s="10" t="n"/>
+      <c r="Z309" s="10" t="n"/>
+      <c r="AA309" s="10" t="n"/>
+      <c r="AB309" s="10" t="n"/>
+      <c r="AC309" s="10" t="n"/>
+      <c r="AD309" s="10" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="10" t="n"/>
@@ -7720,6 +9280,12 @@
       <c r="V310" s="10" t="n"/>
       <c r="W310" s="10" t="n"/>
       <c r="X310" s="10" t="n"/>
+      <c r="Y310" s="10" t="n"/>
+      <c r="Z310" s="10" t="n"/>
+      <c r="AA310" s="10" t="n"/>
+      <c r="AB310" s="10" t="n"/>
+      <c r="AC310" s="10" t="n"/>
+      <c r="AD310" s="10" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="10" t="n"/>
@@ -7746,6 +9312,12 @@
       <c r="V311" s="10" t="n"/>
       <c r="W311" s="10" t="n"/>
       <c r="X311" s="10" t="n"/>
+      <c r="Y311" s="10" t="n"/>
+      <c r="Z311" s="10" t="n"/>
+      <c r="AA311" s="10" t="n"/>
+      <c r="AB311" s="10" t="n"/>
+      <c r="AC311" s="10" t="n"/>
+      <c r="AD311" s="10" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="10" t="n"/>
@@ -7772,6 +9344,12 @@
       <c r="V312" s="10" t="n"/>
       <c r="W312" s="10" t="n"/>
       <c r="X312" s="10" t="n"/>
+      <c r="Y312" s="10" t="n"/>
+      <c r="Z312" s="10" t="n"/>
+      <c r="AA312" s="10" t="n"/>
+      <c r="AB312" s="10" t="n"/>
+      <c r="AC312" s="10" t="n"/>
+      <c r="AD312" s="10" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="5">

</xml_diff>